<commit_message>
PBC pointée sur l'inventaire des nouveaux fichiers du 22/10/2026 ; script d'envoi par lots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261022.xlsx
+++ b/FPPN_PBC_complete_pointee_20261022.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reçus hors liste" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Points à clarifier" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage autres équipes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage nouveaux fichiers" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PBC Actuariat FPPN'!$B$12:$P$12</definedName>
@@ -25,6 +26,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Points à clarifier'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Points à clarifier'!$A$1:$E$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pointage autres équipes'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Pointage nouveaux fichiers'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -1086,7 +1088,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="117" customHeight="1" s="48">
+    <row r="12" ht="192" customHeight="1" s="48">
       <c r="B12" s="70">
         <f>+B11+1</f>
         <v/>
@@ -1108,18 +1110,19 @@
         <v>46316</v>
       </c>
       <c r="I12" s="73" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="J12" s="74" t="n"/>
       <c r="K12" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026. Seuls des fichiers de précomptes ont été reçus : ils ne décrivent pas les prestations.
-Pointage des autres équipes (22/10/2026) : Document intitulé « cartographie des risques » contenant les barèmes des prestations, reçu par l'équipe comptable le 20/10/2026. Copie à obtenir auprès de l'équipe d'audit comptable. Cahier des charges (item 100) toujours attendu.</t>
+Pointage des autres équipes (22/10/2026) : Document intitulé « cartographie des risques » contenant les barèmes des prestations, reçu par l'équipe comptable le 20/10/2026. Copie à obtenir auprès de l'équipe d'audit comptable. Cahier des charges (item 100) toujours attendu.
+Nouveaux fichiers du 22/10/2026 : Règles et barèmes des prestations (maladie, invalidité-décès, EFC, PEP). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ».</t>
         </is>
       </c>
       <c r="M12" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
+          <t>Reçu</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1163,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="192" customHeight="1" s="48">
+    <row r="14" ht="252" customHeight="1" s="48">
       <c r="B14" s="70">
         <f>+B13+1</f>
         <v/>
@@ -1188,7 +1191,8 @@
       <c r="K14" s="75" t="inlineStr">
         <is>
           <t>Convention et avenants : non reçus. Reçu, fichiers de gestion : précomptes retour CGRAE : 30 mois sur 80 (février à mai 2024, juillet 2024 à août 2026) ; manque : janvier 2020 à janvier 2024, juin 2024. Bordereaux : 26 mois sur 80 (février 2024 à septembre 2025, novembre 2025 à janvier 2026, mai à juillet 2026) ; manque : janvier 2020 à janvier 2024, octobre 2025, février à avril 2026, août 2026. Pièces des retraités : 28 mois sur 80 (février 2024 à janvier 2026, mai à août 2026) ; manque : janvier 2020 à janvier 2024, février à avril 2026.
-Pointage des autres équipes (22/10/2026) : Tableau récapitulatif des contrats et conventions (dont CGRAE) reçu partiellement par l'équipe comptable ; liste complète en attente.</t>
+Pointage des autres équipes (22/10/2026) : Tableau récapitulatif des contrats et conventions (dont CGRAE) reçu partiellement par l'équipe comptable ; liste complète en attente.
+Nouveaux fichiers du 22/10/2026 : Convention avec la CGRAE reçue ; avenants à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan, 9 p.).</t>
         </is>
       </c>
       <c r="M14" s="76" t="inlineStr">
@@ -1278,7 +1282,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="72" customHeight="1" s="48">
+    <row r="19" ht="147" customHeight="1" s="48">
       <c r="B19" s="70">
         <f>+B18+1</f>
         <v/>
@@ -1299,17 +1303,20 @@
       <c r="H19" s="73" t="n">
         <v>46318</v>
       </c>
-      <c r="I19" s="73" t="n"/>
+      <c r="I19" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J19" s="74" t="n"/>
       <c r="K19" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Rapports actuariels et calcul des provisions : en attente pour l'équipe comptable également.</t>
+Pointage des autres équipes (22/10/2026) : Rapports actuariels et calcul des provisions : en attente pour l'équipe comptable également.
+Nouveaux fichiers du 22/10/2026 : Études techniques internes reçues ; aucun rapport actuariel ni calcul des provisions. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » ; « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » (.docx, .pdf).</t>
         </is>
       </c>
       <c r="M19" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1662,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="57" customHeight="1" s="48">
+    <row r="34" ht="102" customHeight="1" s="48">
       <c r="B34" s="70">
         <f>+B31+1</f>
         <v/>
@@ -1676,16 +1683,19 @@
       <c r="H34" s="73" t="n">
         <v>46316</v>
       </c>
-      <c r="I34" s="73" t="n"/>
+      <c r="I34" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J34" s="74" t="n"/>
       <c r="K34" s="75" t="inlineStr">
         <is>
-          <t>Non reçu dans l'envoi du 15/10/2026. Les fichiers de versements EFC 870 et PEP 998 reçus ne décrivent pas les règles des produits.</t>
+          <t>Non reçu dans l'envoi du 15/10/2026. Les fichiers de versements EFC 870 et PEP 998 reçus ne décrivent pas les règles des produits.
+Nouveaux fichiers du 22/10/2026 : Description des produits d'épargne EFC et PEP. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ».</t>
         </is>
       </c>
       <c r="M34" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Reçu</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1739,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="33.75" customHeight="1" s="48">
+    <row r="36" ht="102" customHeight="1" s="48">
       <c r="B36" s="70">
         <f>+B35+1</f>
         <v/>
@@ -1750,16 +1760,19 @@
       <c r="H36" s="73" t="n">
         <v>46318</v>
       </c>
-      <c r="I36" s="73" t="n"/>
+      <c r="I36" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J36" s="74" t="n"/>
       <c r="K36" s="75" t="inlineStr">
         <is>
-          <t>Non reçu dans l'envoi du 15/10/2026.</t>
+          <t>Non reçu dans l'envoi du 15/10/2026.
+Nouveaux fichiers du 22/10/2026 : Taux crédité à rechercher dans le manuel et le cahier des charges ; décisions annuelles non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; cahier des charges EFC et PEP 2021.</t>
         </is>
       </c>
       <c r="M36" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1825,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="72" customHeight="1" s="48">
+    <row r="40" ht="162" customHeight="1" s="48">
       <c r="B40" s="70">
         <f>+B37+1</f>
         <v/>
@@ -1833,7 +1846,9 @@
       <c r="H40" s="73" t="n">
         <v>46316</v>
       </c>
-      <c r="I40" s="73" t="n"/>
+      <c r="I40" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J40" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -1842,12 +1857,13 @@
       <c r="K40" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : État des placements, dossiers des DAT et tableau de synthèse en attente pour l'équipe comptable également.</t>
+Pointage des autres équipes (22/10/2026) : État des placements, dossiers des DAT et tableau de synthèse en attente pour l'équipe comptable également.
+Nouveaux fichiers du 22/10/2026 : États de rapprochement bancaire 2020 à 2026 reçus ; échéancier des placements (DAT, FCP) non reçu. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » (onglets par banque : BOA PEP, BOA EFC, BOA BF, BOA FPPN, ORABANK, BANQUE ATLANTIQUE).</t>
         </is>
       </c>
       <c r="M40" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1941,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="57" customHeight="1" s="48">
+    <row r="43" ht="117" customHeight="1" s="48">
       <c r="B43" s="70">
         <f>+B42+1</f>
         <v/>
@@ -1946,17 +1962,20 @@
       <c r="H43" s="73" t="n">
         <v>46323</v>
       </c>
-      <c r="I43" s="73" t="n"/>
+      <c r="I43" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J43" s="74" t="n"/>
       <c r="K43" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Dossiers des programmes immobiliers en attente (liste des immeubles : M. Koffi).</t>
+Pointage des autres équipes (22/10/2026) : Dossiers des programmes immobiliers en attente (liste des immeubles : M. Koffi).
+Nouveaux fichiers du 22/10/2026 : Titres et baux reçus ; valeurs et dernières évaluations non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : certificats de propriété, acte de vente, « CONTRAT DE BAIL SONAPIE N° 2124-03002 / 03037 FPPN.pdf ».</t>
         </is>
       </c>
       <c r="M43" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="72" customHeight="1" s="48">
+    <row r="48" ht="147" customHeight="1" s="48">
       <c r="B48" s="70">
         <f>+B47+1</f>
         <v/>
@@ -2059,17 +2078,20 @@
       <c r="H48" s="73" t="n">
         <v>46316</v>
       </c>
-      <c r="I48" s="73" t="n"/>
+      <c r="I48" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J48" s="74" t="n"/>
       <c r="K48" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Organigramme 2022 (identité et postes) reçu partiellement par l'équipe comptable ; version numérique en attente.</t>
+Pointage des autres équipes (22/10/2026) : Organigramme 2022 (identité et postes) reçu partiellement par l'équipe comptable ; version numérique en attente.
+Nouveaux fichiers du 22/10/2026 : Organigrammes 2020 et 2021 et un courrier de nomination reçus ; contacts des responsables non reçus. Contenu à analyser. Fichiers : « ORGANIGRAMME FPPN 2021(1).pdf » ; 03-Nouveaux Juridiques : « OrganigrammeFPPN_ORI (A) 2020.docx » ; « COURRIER DE NOMINATION DÉFINITIVE.pdf ».</t>
         </is>
       </c>
       <c r="M48" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -2083,7 +2105,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="42" customHeight="1" s="48">
+    <row r="51" ht="117" customHeight="1" s="48">
       <c r="B51" s="70">
         <f>+B48+1</f>
         <v/>
@@ -2104,7 +2126,9 @@
       <c r="H51" s="73" t="n">
         <v>46316</v>
       </c>
-      <c r="I51" s="73" t="n"/>
+      <c r="I51" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J51" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -2112,12 +2136,13 @@
       </c>
       <c r="K51" s="75" t="inlineStr">
         <is>
-          <t>Non reçu dans l'envoi du 15/10/2026.</t>
+          <t>Non reçu dans l'envoi du 15/10/2026.
+Nouveaux fichiers du 22/10/2026 : Sinistralité observée par le FPPN (au 30 juin, historique 2015 à 2021) et interprétation : méthode du FPPN à confronter à la formule de la Décision n° 05/2022. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » (onglets Tableau, Notes, Historique 2015-2021) ; « INTERPRETATION DES RATIOS… » (.docx, .pdf).</t>
         </is>
       </c>
       <c r="M51" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -2201,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="87" customFormat="1" customHeight="1" s="68">
+    <row r="54" ht="147" customFormat="1" customHeight="1" s="68">
       <c r="B54" s="70">
         <f>+B53+1</f>
         <v/>
@@ -2229,7 +2254,8 @@
       <c r="K54" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Barèmes en vigueur reçus dans la « cartographie des risques » (20/10/2026). Barèmes successifs depuis 2001 et décisions non reçus. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Barèmes en vigueur reçus dans la « cartographie des risques » (20/10/2026). Barèmes successifs depuis 2001 et décisions non reçus. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Barèmes 2021 reçus ; barèmes successifs depuis 2001 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : cartographie des risques.</t>
         </is>
       </c>
       <c r="M54" s="76" t="inlineStr">
@@ -2310,7 +2336,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="72" customHeight="1" s="48">
+    <row r="57" ht="147" customHeight="1" s="48">
       <c r="B57" s="70">
         <f>+B56+1</f>
         <v/>
@@ -2331,21 +2357,24 @@
       <c r="H57" s="73" t="n">
         <v>46316</v>
       </c>
-      <c r="I57" s="73" t="n"/>
+      <c r="I57" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J57" s="74" t="n"/>
       <c r="K57" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Liste des pièces du dossier d'allocation décès et conditions d'octroi en attente (M. Soumahoro).</t>
+Pointage des autres équipes (22/10/2026) : Liste des pièces du dossier d'allocation décès et conditions d'octroi en attente (M. Soumahoro).
+Nouveaux fichiers du 22/10/2026 : Listes des pièces exigées pour les prestations décès ; cahier des charges reçu (item 100). Fichiers : 05-Nouveaux Prestations : « Liste des pièces à fournir en cas de décès d'un membre participant.pdf », « … d'un ayant-droit.pdf », « … pour les frais funeraires.pdf ».</t>
         </is>
       </c>
       <c r="M57" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="87" customHeight="1" s="48">
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="147" customHeight="1" s="48">
       <c r="B58" s="70">
         <f>+B57+1</f>
         <v/>
@@ -2373,7 +2402,8 @@
       <c r="K58" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Manuels de procédures (adhésions, cotisations, prestations, crédits) reçus non signés par l'équipe comptable ; versions signées à transmettre. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Manuels de procédures (adhésions, cotisations, prestations, crédits) reçus non signés par l'équipe comptable ; versions signées à transmettre. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Documents décrivant le traitement des prestations. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » ; listes des pièces décès.</t>
         </is>
       </c>
       <c r="M58" s="76" t="inlineStr">
@@ -2731,7 +2761,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="102" customHeight="1" s="48">
+    <row r="72" ht="177" customHeight="1" s="48">
       <c r="B72" s="70">
         <f>+B69+1</f>
         <v/>
@@ -2757,7 +2787,8 @@
       <c r="K72" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
-Pointage des autres équipes (22/10/2026) : Actes d'agrément et correspondances avec l'AIRMS reçus en version papier par l'équipe comptable ; version numérique en attente. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Actes d'agrément et correspondances avec l'AIRMS reçus en version papier par l'équipe comptable ; version numérique en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Attestation d'immatriculation n° 1D/0052016/CI du 05/04/2017 reçue ; décision d'agrément et liste des risques autorisés à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « NUMERO D'IMMATRICULATION AIRSM N° 1D-0052016-CI DU 05-04-2017.pdf » (scan).</t>
         </is>
       </c>
       <c r="M72" s="76" t="inlineStr">
@@ -2803,7 +2834,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="42" customHeight="1" s="48">
+    <row r="74" ht="102" customHeight="1" s="48">
       <c r="B74" s="70">
         <f>+B73+1</f>
         <v/>
@@ -2824,20 +2855,23 @@
       <c r="H74" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I74" s="73" t="n"/>
+      <c r="I74" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J74" s="74" t="n"/>
       <c r="K74" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).</t>
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
+Nouveaux fichiers du 22/10/2026 : Règlement du PEP et de l'EFC. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ».</t>
         </is>
       </c>
       <c r="M74" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="87" customHeight="1" s="48">
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="177" customHeight="1" s="48">
       <c r="B75" s="70">
         <f>+B74+1</f>
         <v/>
@@ -2858,17 +2892,20 @@
       <c r="H75" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I75" s="73" t="n"/>
+      <c r="I75" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J75" s="74" t="n"/>
       <c r="K75" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
-Pointage des autres équipes (22/10/2026) : États financiers reçus par l'équipe comptable. Rapports du commissaire aux comptes 2022 à 2025 en attente, 2020 et 2021 à retrouver par le FPPN.</t>
+Pointage des autres équipes (22/10/2026) : États financiers reçus par l'équipe comptable. Rapports du commissaire aux comptes 2022 à 2025 en attente, 2020 et 2021 à retrouver par le FPPN.
+Nouveaux fichiers du 22/10/2026 : États financiers 2020 au 31/08/2026 reçus ; rapports du commissaire aux comptes et états par risque long non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf », « ETATS FINANCIERS AU 31-08-2026.pdf » (scans) ; « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf ».</t>
         </is>
       </c>
       <c r="M75" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2978,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="87" customHeight="1" s="48">
+    <row r="78" ht="147" customHeight="1" s="48">
       <c r="B78" s="70">
         <f>+B77+1</f>
         <v/>
@@ -2969,7 +3006,8 @@
       <c r="K78" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
-Pointage des autres équipes (22/10/2026) : PV d'AG reçus par l'équipe comptable sauf 2020 et 2023 : l'affectation de 2023 reste à obtenir. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : PV d'AG reçus par l'équipe comptable sauf 2020 et 2023 : l'affectation de 2023 reste à obtenir. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : AG du 15/02/2024 : affectation à vérifier ; origine du compte 10620000 non documentée. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan).</t>
         </is>
       </c>
       <c r="M78" s="76" t="inlineStr">
@@ -3046,7 +3084,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="87" customHeight="1" s="48">
+    <row r="81" ht="162" customHeight="1" s="48">
       <c r="B81" s="70">
         <f>+B80+1</f>
         <v/>
@@ -3074,7 +3112,8 @@
       <c r="K81" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
-Pointage des autres équipes (22/10/2026) : Procès-verbaux des AG, CA et commissions reçus par l'équipe comptable, sauf 2020 et 2023. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Procès-verbaux des AG, CA et commissions reçus par l'équipe comptable, sauf 2020 et 2023. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : PV de 2024 et compositions des organes reçus ; calendrier statutaire et autres PV à compléter. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » ; listes des administrateurs et membres de la commission de surveillance.</t>
         </is>
       </c>
       <c r="M81" s="76" t="inlineStr">
@@ -3199,7 +3238,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="57" customHeight="1" s="48">
+    <row r="87" ht="102" customHeight="1" s="48">
       <c r="B87" s="70">
         <f>+B86+1</f>
         <v/>
@@ -3220,7 +3259,9 @@
       <c r="H87" s="73" t="n">
         <v>46317</v>
       </c>
-      <c r="I87" s="73" t="n"/>
+      <c r="I87" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J87" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -3228,12 +3269,13 @@
       </c>
       <c r="K87" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de l'entretien du 19/10/2026 avec le responsable des cotisations (PBC complémentaire cotisations).</t>
+          <t>Demande issue de l'entretien du 19/10/2026 avec le responsable des cotisations (PBC complémentaire cotisations).
+Nouveaux fichiers du 22/10/2026 : EFC, PEP et Grenier documentés ; MEDOC et flotte automobile non documentés. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne, cahiers des charges 2021, « POLITIK DE CREDIT DU GRENIER VFVF.doc ».</t>
         </is>
       </c>
       <c r="M87" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -3842,7 +3884,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="102" customHeight="1" s="48">
+    <row r="106" ht="147" customHeight="1" s="48">
       <c r="B106" s="70">
         <f>+B105+1</f>
         <v/>
@@ -3864,18 +3906,19 @@
         <v>46321</v>
       </c>
       <c r="I106" s="73" t="n">
-        <v>46310</v>
+        <v>46317</v>
       </c>
       <c r="J106" s="74" t="n"/>
       <c r="K106" s="75" t="inlineStr">
         <is>
           <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
-Pointage des autres équipes (22/10/2026) : Règlement des crédits reçu ; aucune politique écrite de dépréciation (le FPPN cite les garanties et un taux de 1 %). Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Règlement des crédits reçu ; aucune politique écrite de dépréciation (le FPPN cite les garanties et un taux de 1 %). Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Politique de crédit du Grenier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « POLITIK DE CREDIT DU GRENIER VFVF.doc ».</t>
         </is>
       </c>
       <c r="M106" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
+          <t>Reçu</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3960,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="72" customHeight="1" s="48">
+    <row r="108" ht="177" customHeight="1" s="48">
       <c r="B108" s="70">
         <f>+B107+1</f>
         <v/>
@@ -3938,7 +3981,9 @@
       <c r="H108" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I108" s="73" t="n"/>
+      <c r="I108" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J108" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -3947,12 +3992,13 @@
       <c r="K108" s="75" t="inlineStr">
         <is>
           <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
-Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi).</t>
+Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi).
+Nouveaux fichiers du 22/10/2026 : Les DISA donnent, pour chaque salarié déclaré à la CNPS, l'année de naissance, la date d'embauche et le salaire brut annuel : base possible de la provision pour départ à la retraite. Situation au 31/08/2026 non reçue. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « DISA_256927_2021.xls » à « DISA_256927_2025.xls » (colonnes ANNEE NAISS., DATE EMBAUCHE, DATE DEPART, SALAIRE BRUT).</t>
         </is>
       </c>
       <c r="M108" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4115,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="72" customHeight="1" s="48">
+    <row r="114" ht="132" customHeight="1" s="48">
       <c r="B114" s="70">
         <f>+B111+1</f>
         <v/>
@@ -4090,7 +4136,9 @@
       <c r="H114" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I114" s="73" t="n"/>
+      <c r="I114" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J114" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -4099,12 +4147,13 @@
       <c r="K114" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Dossiers des DAT en attente pour l'équipe comptable également.</t>
+Pointage des autres équipes (22/10/2026) : Dossiers des DAT en attente pour l'équipe comptable également.
+Nouveaux fichiers du 22/10/2026 : Mouvements des comptes BOA à lire ; conventions et relevés du DAT non reçus. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : états de rapprochement bancaire 2020 à 2026.</t>
         </is>
       </c>
       <c r="M114" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4185,7 +4234,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="42" customHeight="1" s="48">
+    <row r="117" ht="102" customHeight="1" s="48">
       <c r="B117" s="70">
         <f>+B116+1</f>
         <v/>
@@ -4206,20 +4255,23 @@
       <c r="H117" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I117" s="73" t="n"/>
+      <c r="I117" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J117" s="74" t="n"/>
       <c r="K117" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Nouveaux fichiers du 22/10/2026 : La convention doit préciser la dénomination et le statut de la structure CMP. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf ».</t>
         </is>
       </c>
       <c r="M117" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="72" customHeight="1" s="48">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="162" customHeight="1" s="48">
       <c r="B118" s="70">
         <f>+B117+1</f>
         <v/>
@@ -4240,17 +4292,20 @@
       <c r="H118" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I118" s="73" t="n"/>
+      <c r="I118" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J118" s="74" t="n"/>
       <c r="K118" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Titres de propriété et tableau de synthèse des biens en attente (M. Sangaré).</t>
+Pointage des autres équipes (22/10/2026) : Titres de propriété et tableau de synthèse des biens en attente (M. Sangaré).
+Nouveaux fichiers du 22/10/2026 : Deux certificats de propriété et un acte de vente reçus ; situation de chaque terrain (projet, attribution, litige) non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « Certificat de Propriété Terrain Marcori (Siège).pdf » ; « Certificat de Propriété Terrain Plateau.pdf » ; « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE… ».</t>
         </is>
       </c>
       <c r="M118" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4411,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="42" customHeight="1" s="48">
+    <row r="122" ht="102" customHeight="1" s="48">
       <c r="B122" s="70">
         <f>+B121+1</f>
         <v/>
@@ -4377,7 +4432,9 @@
       <c r="H122" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I122" s="73" t="n"/>
+      <c r="I122" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J122" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -4385,12 +4442,13 @@
       </c>
       <c r="K122" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Nouveaux fichiers du 22/10/2026 : Convention de la clinique (CMP) avec Transvie reçue ; bilan d'ouverture et détail des comptes 47111104 et 47111105 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf » (scan).</t>
         </is>
       </c>
       <c r="M122" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4487,7 @@
         </is>
       </c>
     </row>
-    <row r="124" ht="102" customHeight="1" s="48">
+    <row r="124" ht="162" customHeight="1" s="48">
       <c r="B124" s="70">
         <f>+B123+1</f>
         <v/>
@@ -4451,7 +4509,7 @@
         <v>46321</v>
       </c>
       <c r="I124" s="73" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="J124" s="74" t="inlineStr">
         <is>
@@ -4461,12 +4519,13 @@
       <c r="K124" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Liste des comptes bancaires reçue partiellement par l'équipe comptable ; liste par exercice en attente. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Liste des comptes bancaires reçue partiellement par l'équipe comptable ; liste par exercice en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Liste des comptes bancaires et habilitations de signature. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « LISTE DES COMPTES BANCAIRES  DU FPPN.pdf » ; « Habilitation de signatures.pdf » (scans).</t>
         </is>
       </c>
       <c r="M124" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
+          <t>Reçu</t>
         </is>
       </c>
     </row>
@@ -4556,7 +4615,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="102" customHeight="1" s="48">
+    <row r="129" ht="162" customHeight="1" s="48">
       <c r="B129" s="70">
         <f>+B128+1</f>
         <v/>
@@ -4584,7 +4643,8 @@
       <c r="K129" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : Barèmes des prestations reçus dans la « cartographie des risques » (20/10/2026), à confronter au barème par grade demandé. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Barèmes des prestations reçus dans la « cartographie des risques » (20/10/2026), à confronter au barème par grade demandé. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Barème des allocations décès par grade à lire dans le cahier des charges 2021. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».</t>
         </is>
       </c>
       <c r="M129" s="76" t="inlineStr">
@@ -4696,7 +4756,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="87" customHeight="1" s="48">
+    <row r="133" ht="162" customHeight="1" s="48">
       <c r="B133" s="70">
         <f>+B132+1</f>
         <v/>
@@ -4728,7 +4788,8 @@
       <c r="K133" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Pointage des autres équipes (22/10/2026) : DISA et état 301 reçus sauf 2026 ; ITS et FDFP reçus (2021 manquant) ; déclarations CNPS en attente. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : DISA et état 301 reçus sauf 2026 ; ITS et FDFP reçus (2021 manquant) ; déclarations CNPS en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025.</t>
         </is>
       </c>
       <c r="M133" s="76" t="inlineStr">
@@ -4776,7 +4837,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="42" customHeight="1" s="48">
+    <row r="135" ht="102" customHeight="1" s="48">
       <c r="B135" s="70">
         <f>+B134+1</f>
         <v/>
@@ -4797,16 +4858,19 @@
       <c r="H135" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I135" s="73" t="n"/>
+      <c r="I135" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J135" s="74" t="n"/>
       <c r="K135" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Nouveaux fichiers du 22/10/2026 : Taux servi de 3,5 % à vérifier dans ces documents ; décision non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne ; cahier des charges EFC et PEP 2021.</t>
         </is>
       </c>
       <c r="M135" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4882,7 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="42" customHeight="1" s="48">
+    <row r="138" ht="117" customHeight="1" s="48">
       <c r="B138" s="70">
         <f>+B135+1</f>
         <v/>
@@ -4839,7 +4903,9 @@
       <c r="H138" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I138" s="73" t="n"/>
+      <c r="I138" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J138" s="74" t="inlineStr">
         <is>
           <t>Physique et Electronique</t>
@@ -4847,16 +4913,17 @@
       </c>
       <c r="K138" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).</t>
+          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
+Nouveaux fichiers du 22/10/2026 : Cahiers des charges du régime des prestations sociales, version 2021. Versions antérieures à 2021 non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (17 p.) ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » (10 p.).</t>
         </is>
       </c>
       <c r="M138" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="102" customHeight="1" s="48">
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="162" customHeight="1" s="48">
       <c r="B139" s="70">
         <f>+B138+1</f>
         <v/>
@@ -4888,7 +4955,8 @@
       <c r="K139" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : Barèmes des prestations reçus dans la « cartographie des risques » (20/10/2026) ; tableau des allocations officiel non identifié. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Barèmes des prestations reçus dans la « cartographie des risques » (20/10/2026) ; tableau des allocations officiel non identifié. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : Le tableau des allocations doit figurer dans le cahier des charges 2021 ; versions 2020 et postérieures à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».</t>
         </is>
       </c>
       <c r="M139" s="76" t="inlineStr">
@@ -4897,7 +4965,7 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="87" customHeight="1" s="48">
+    <row r="140" ht="132" customHeight="1" s="48">
       <c r="B140" s="70">
         <f>+B139+1</f>
         <v/>
@@ -4918,7 +4986,9 @@
       <c r="H140" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I140" s="73" t="n"/>
+      <c r="I140" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J140" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -4927,12 +4997,13 @@
       <c r="K140" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : À rechercher dans les manuels de procédures non signés reçus par l'équipe comptable le 21/10/2026.</t>
+Pointage des autres équipes (22/10/2026) : À rechercher dans les manuels de procédures non signés reçus par l'équipe comptable le 21/10/2026.
+Nouveaux fichiers du 22/10/2026 : Manuel des produits d'épargne (PEP et EFC). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ».</t>
         </is>
       </c>
       <c r="M140" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Reçu</t>
         </is>
       </c>
     </row>
@@ -4944,7 +5015,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="87" customHeight="1" s="48">
+    <row r="143" ht="162" customHeight="1" s="48">
       <c r="B143" s="70">
         <f>+B140+1</f>
         <v/>
@@ -4965,7 +5036,9 @@
       <c r="H143" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I143" s="73" t="n"/>
+      <c r="I143" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J143" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -4974,12 +5047,13 @@
       <c r="K143" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi) : le statut civil ou policier devra y figurer.</t>
+Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi) : le statut civil ou policier devra y figurer.
+Nouveaux fichiers du 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS (personnel civil) ; les fonctionnaires de police en service n'y figurent a priori pas. Statut à confirmer. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : DISA 2021 à 2025 ; « RECAPSALAIRES » des états 301.</t>
         </is>
       </c>
       <c r="M143" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5169,7 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="87" customHeight="1" s="48">
+    <row r="149" ht="147" customHeight="1" s="48">
       <c r="B149" s="70">
         <f>+B148+1</f>
         <v/>
@@ -5123,7 +5197,8 @@
       <c r="K149" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : PV d'AG reçus par l'équipe comptable, sauf 2020 et 2023 ; affectations des résultats à y vérifier. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : PV d'AG reçus par l'équipe comptable, sauf 2020 et 2023 ; affectations des résultats à y vérifier. Copie à obtenir auprès de l'équipe d'audit comptable.
+Nouveaux fichiers du 22/10/2026 : PV de l'AG ordinaire du 15/02/2024 reçu ; autres AG d'affectation non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan).</t>
         </is>
       </c>
       <c r="M149" s="76" t="inlineStr">
@@ -5316,7 +5391,7 @@
       </c>
       <c r="D6" s="95" t="inlineStr">
         <is>
-          <t>45, 70</t>
+          <t>2, 16, 33, 45, 46, 70, 74, 90, 100, 102</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5407,7 @@
       </c>
       <c r="D7" s="95" t="inlineStr">
         <is>
-          <t>1, 2, 3, 4, 6, 8, 9, 12, 13, 17, 21, 28, 30, 34, 35, 37, 42, 44, 50, 53, 71, 73, 74, 90, 93, 97, 101, 107</t>
+          <t>1, 3, 4, 6, 7, 8, 9, 12, 13, 17, 18, 20, 21, 23, 26, 27, 28, 30, 34, 35, 37, 42, 44, 47, 50, 53, 57, 71, 73, 76, 80, 83, 84, 88, 93, 97, 99, 101, 103, 107</t>
         </is>
       </c>
     </row>
@@ -5348,7 +5423,7 @@
       </c>
       <c r="D8" s="95" t="inlineStr">
         <is>
-          <t>5, 7, 10, 11, 14, 15, 16, 18, 19, 20, 22, 23, 24, 25, 26, 27, 29, 31, 32, 33, 36, 38, 39, 40, 41, 43, 46, 47, 48, 49, 51, 52, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 72, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 91, 92, 94, 95, 96, 98, 99, 100, 102, 103, 104, 105, 106, 108, 109</t>
+          <t>5, 10, 11, 14, 15, 19, 22, 24, 25, 29, 31, 32, 36, 38, 39, 40, 41, 43, 48, 49, 51, 52, 54, 55, 56, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 72, 75, 77, 78, 79, 81, 82, 85, 86, 87, 89, 91, 92, 94, 95, 96, 98, 104, 105, 106, 108, 109</t>
         </is>
       </c>
     </row>
@@ -45196,4 +45271,1066 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:G38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" style="48" min="2" max="2"/>
+    <col width="48" customWidth="1" style="48" min="3" max="3"/>
+    <col width="16" customWidth="1" style="48" min="4" max="4"/>
+    <col width="16" customWidth="1" style="48" min="5" max="5"/>
+    <col width="60" customWidth="1" style="48" min="6" max="6"/>
+    <col width="60" customWidth="1" style="48" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="97" t="inlineStr">
+        <is>
+          <t>Pointage sur les nouveaux fichiers reçus le 22/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1" s="48">
+      <c r="B3" s="79" t="inlineStr">
+        <is>
+          <t>Source : « FPPN_inventaire_nouveaux_fichiers_20261022.xlsx » (113 fichiers). Pointage fondé sur le nom, la taille et la première page lisible de chaque fichier : le contenu reste à analyser. Un statut n'est jamais abaissé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="80" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C5" s="80" t="inlineStr">
+        <is>
+          <t>Document demandé (PBC actuarielle)</t>
+        </is>
+      </c>
+      <c r="D5" s="80" t="inlineStr">
+        <is>
+          <t>Statut avant</t>
+        </is>
+      </c>
+      <c r="E5" s="80" t="inlineStr">
+        <is>
+          <t>Statut après</t>
+        </is>
+      </c>
+      <c r="F5" s="80" t="inlineStr">
+        <is>
+          <t>Fichiers reçus</t>
+        </is>
+      </c>
+      <c r="G5" s="80" t="inlineStr">
+        <is>
+          <t>Commentaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1" s="48">
+      <c r="B6" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="95" t="inlineStr">
+        <is>
+          <t>Règlement ou fiche descriptive de chaque prestation servie (allocation décès, invalidité, prise en charge des retraités, santé, épargne, autres aides) : bénéfic</t>
+        </is>
+      </c>
+      <c r="D6" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E6" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F6" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx »</t>
+        </is>
+      </c>
+      <c r="G6" s="95" t="inlineStr">
+        <is>
+          <t>Règles et barèmes des prestations (maladie, invalidité-décès, EFC, PEP). Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1" s="48">
+      <c r="B7" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="95" t="inlineStr">
+        <is>
+          <t>Convention conclue avec la CGRAE pour la prise en charge des retraités, et ses avenants.</t>
+        </is>
+      </c>
+      <c r="D7" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E7" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F7" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan, 9 p.)</t>
+        </is>
+      </c>
+      <c r="G7" s="95" t="inlineStr">
+        <is>
+          <t>Convention avec la CGRAE reçue ; avenants à vérifier. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1" s="48">
+      <c r="B8" s="96" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>Tout rapport actuariel, étude technique ou note de calcul des engagements envers les mutualistes existant, quelle que soit sa date.</t>
+        </is>
+      </c>
+      <c r="D8" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E8" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » ; « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » (.docx, .pdf)</t>
+        </is>
+      </c>
+      <c r="G8" s="95" t="inlineStr">
+        <is>
+          <t>Études techniques internes reçues ; aucun rapport actuariel ni calcul des provisions. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1" s="48">
+      <c r="B9" s="96" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" s="95" t="inlineStr">
+        <is>
+          <t>Description des produits d'épargne (épargne de fin de carrière, Plan Épargne Plus, autres) : règles de versement, taux d'intérêt servi ou garanti, conditions de</t>
+        </is>
+      </c>
+      <c r="D9" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E9" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F9" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf »</t>
+        </is>
+      </c>
+      <c r="G9" s="95" t="inlineStr">
+        <is>
+          <t>Description des produits d'épargne EFC et PEP. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1" s="48">
+      <c r="B10" s="96" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" s="95" t="inlineStr">
+        <is>
+          <t>Taux d'intérêt crédité sur l'épargne chaque année et décision qui l'a fixé.</t>
+        </is>
+      </c>
+      <c r="D10" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E10" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F10" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; cahier des charges EFC et PEP 2021</t>
+        </is>
+      </c>
+      <c r="G10" s="95" t="inlineStr">
+        <is>
+          <t>Taux crédité à rechercher dans le manuel et le cahier des charges ; décisions annuelles non reçues. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="75" customHeight="1" s="48">
+      <c r="B11" s="96" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" s="95" t="inlineStr">
+        <is>
+          <t>Échéancier des placements au 31/12/2025 et au 31/08/2026 : nature, établissement, montant, date de souscription, date d'échéance, taux, conditions de sortie ant</t>
+        </is>
+      </c>
+      <c r="D11" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E11" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F11" s="95" t="inlineStr">
+        <is>
+          <t>07-Nouveaux Trésorerie et placements : « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » (onglets par banque : BOA PEP, BOA EFC, BOA BF, BOA FPPN, ORABANK, BANQUE ATLANTIQUE)</t>
+        </is>
+      </c>
+      <c r="G11" s="95" t="inlineStr">
+        <is>
+          <t>États de rapprochement bancaire 2020 à 2026 reçus ; échéancier des placements (DAT, FCP) non reçu. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="75" customHeight="1" s="48">
+      <c r="B12" s="96" t="n">
+        <v>23</v>
+      </c>
+      <c r="C12" s="95" t="inlineStr">
+        <is>
+          <t>Biens immobiliers et participations (centre médical, programme immobilier, autres) au 31/08/2026 : valeur au bilan, dernière évaluation, revenus annuels, contra</t>
+        </is>
+      </c>
+      <c r="D12" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E12" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F12" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : certificats de propriété, acte de vente, « CONTRAT DE BAIL SONAPIE N° 2124-03002 / 03037 FPPN.pdf »</t>
+        </is>
+      </c>
+      <c r="G12" s="95" t="inlineStr">
+        <is>
+          <t>Titres et baux reçus ; valeurs et dernières évaluations non reçues. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="75" customHeight="1" s="48">
+      <c r="B13" s="96" t="n">
+        <v>26</v>
+      </c>
+      <c r="C13" s="95" t="inlineStr">
+        <is>
+          <t>Nom, fonction et contact des responsables à rencontrer pour les prestations, l'épargne, les placements et les données des mutualistes.</t>
+        </is>
+      </c>
+      <c r="D13" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E13" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F13" s="95" t="inlineStr">
+        <is>
+          <t>« ORGANIGRAMME FPPN 2021(1).pdf » ; 03-Nouveaux Juridiques : « OrganigrammeFPPN_ORI (A) 2020.docx » ; « COURRIER DE NOMINATION DÉFINITIVE.pdf »</t>
+        </is>
+      </c>
+      <c r="G13" s="95" t="inlineStr">
+        <is>
+          <t>Organigrammes 2020 et 2021 et un courrier de nomination reçus ; contacts des responsables non reçus. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="75" customHeight="1" s="48">
+      <c r="B14" s="96" t="n">
+        <v>27</v>
+      </c>
+      <c r="C14" s="95" t="inlineStr">
+        <is>
+          <t>Fichiers de suivi de la sinistralité de 2019 au 31/08/2026 (tableau de bord du service), avec le détail du calcul du taux de sinistralité.</t>
+        </is>
+      </c>
+      <c r="D14" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E14" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F14" s="95" t="inlineStr">
+        <is>
+          <t>05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » (onglets Tableau, Notes, Historique 2015-2021) ; « INTERPRETATION DES RATIOS… » (.docx, .pdf)</t>
+        </is>
+      </c>
+      <c r="G14" s="95" t="inlineStr">
+        <is>
+          <t>Sinistralité observée par le FPPN (au 30 juin, historique 2015 à 2021) et interprétation : méthode du FPPN à confronter à la formule de la Décision n° 05/2022. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="75" customHeight="1" s="48">
+      <c r="B15" s="96" t="n">
+        <v>30</v>
+      </c>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>Barèmes successifs des capitaux décès, frais funéraires et allocations aux ayants droit, de 2001 à 2026, avec les décisions qui les ont adoptés.</t>
+        </is>
+      </c>
+      <c r="D15" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E15" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F15" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : cartographie des risques</t>
+        </is>
+      </c>
+      <c r="G15" s="95" t="inlineStr">
+        <is>
+          <t>Barèmes 2021 reçus ; barèmes successifs depuis 2001 non reçus. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="75" customHeight="1" s="48">
+      <c r="B16" s="96" t="n">
+        <v>33</v>
+      </c>
+      <c r="C16" s="95" t="inlineStr">
+        <is>
+          <t>Liste des pièces exigées pour chaque prestation et cahier du régime des prestations sociales.</t>
+        </is>
+      </c>
+      <c r="D16" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E16" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F16" s="95" t="inlineStr">
+        <is>
+          <t>05-Nouveaux Prestations : « Liste des pièces à fournir en cas de décès d'un membre participant.pdf », « … d'un ayant-droit.pdf », « … pour les frais funeraires.pdf »</t>
+        </is>
+      </c>
+      <c r="G16" s="95" t="inlineStr">
+        <is>
+          <t>Listes des pièces exigées pour les prestations décès ; cahier des charges reçu (item 100).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="75" customHeight="1" s="48">
+      <c r="B17" s="96" t="n">
+        <v>34</v>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
+        <is>
+          <t>Projet de manuel de procédures de 2014 et tout document décrivant le traitement des prestations.</t>
+        </is>
+      </c>
+      <c r="D17" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E17" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F17" s="95" t="inlineStr">
+        <is>
+          <t>05-Nouveaux Prestations : « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » ; listes des pièces décès</t>
+        </is>
+      </c>
+      <c r="G17" s="95" t="inlineStr">
+        <is>
+          <t>Documents décrivant le traitement des prestations. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="75" customHeight="1" s="48">
+      <c r="B18" s="96" t="n">
+        <v>44</v>
+      </c>
+      <c r="C18" s="95" t="inlineStr">
+        <is>
+          <t>Décision d'agrément du FPPN, numéro et attestation d'immatriculation au registre national, avec la liste des risques autorisés (règlement n° 07/2009, art. 22).</t>
+        </is>
+      </c>
+      <c r="D18" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E18" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F18" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « NUMERO D'IMMATRICULATION AIRSM N° 1D-0052016-CI DU 05-04-2017.pdf » (scan)</t>
+        </is>
+      </c>
+      <c r="G18" s="95" t="inlineStr">
+        <is>
+          <t>Attestation d'immatriculation n° 1D/0052016/CI du 05/04/2017 reçue ; décision d'agrément et liste des risques autorisés à vérifier. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="75" customHeight="1" s="48">
+      <c r="B19" s="96" t="n">
+        <v>46</v>
+      </c>
+      <c r="C19" s="95" t="inlineStr">
+        <is>
+          <t>Règlement des produits PEP et EFC : conditions de retrait, échéances, âge de versement, taux servi.</t>
+        </is>
+      </c>
+      <c r="D19" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E19" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F19" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf »</t>
+        </is>
+      </c>
+      <c r="G19" s="95" t="inlineStr">
+        <is>
+          <t>Règlement du PEP et de l'EFC. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="75" customHeight="1" s="48">
+      <c r="B20" s="96" t="n">
+        <v>47</v>
+      </c>
+      <c r="C20" s="95" t="inlineStr">
+        <is>
+          <t>Rapports du commissaire aux comptes 2020 à 2025 et états financiers par risque long (règlement d'exécution n° 004/2022, art. 12 et 13).</t>
+        </is>
+      </c>
+      <c r="D20" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E20" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F20" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf », « ETATS FINANCIERS AU 31-08-2026.pdf » (scans) ; « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf »</t>
+        </is>
+      </c>
+      <c r="G20" s="95" t="inlineStr">
+        <is>
+          <t>États financiers 2020 au 31/08/2026 reçus ; rapports du commissaire aux comptes et états par risque long non reçus. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="75" customHeight="1" s="48">
+      <c r="B21" s="96" t="n">
+        <v>50</v>
+      </c>
+      <c r="C21" s="95" t="inlineStr">
+        <is>
+          <t>PV d'AG d'affectation des excédents 2023 à 2025 et origine du compte 10620000 « Réserve disponible ».</t>
+        </is>
+      </c>
+      <c r="D21" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E21" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F21" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan)</t>
+        </is>
+      </c>
+      <c r="G21" s="95" t="inlineStr">
+        <is>
+          <t>AG du 15/02/2024 : affectation à vérifier ; origine du compte 10620000 non documentée. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="75" customHeight="1" s="48">
+      <c r="B22" s="96" t="n">
+        <v>53</v>
+      </c>
+      <c r="C22" s="95" t="inlineStr">
+        <is>
+          <t>Calendrier statutaire et PV des réunions du conseil, de l'organe de contrôle et de l'AG, 2022 à 2025.</t>
+        </is>
+      </c>
+      <c r="D22" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E22" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F22" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » ; listes des administrateurs et membres de la commission de surveillance</t>
+        </is>
+      </c>
+      <c r="G22" s="95" t="inlineStr">
+        <is>
+          <t>PV de 2024 et compositions des organes reçus ; calendrier statutaire et autres PV à compléter. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="75" customHeight="1" s="48">
+      <c r="B23" s="96" t="n">
+        <v>57</v>
+      </c>
+      <c r="C23" s="95" t="inlineStr">
+        <is>
+          <t>Documentation de chaque produit : EFC, PEP, MEDOC, prêts du Grenier, flotte automobile (règlement, conditions de souscription, montants, conditions de sortie et</t>
+        </is>
+      </c>
+      <c r="D23" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E23" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F23" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : manuel de produit d'épargne, cahiers des charges 2021, « POLITIK DE CREDIT DU GRENIER VFVF.doc »</t>
+        </is>
+      </c>
+      <c r="G23" s="95" t="inlineStr">
+        <is>
+          <t>EFC, PEP et Grenier documentés ; MEDOC et flotte automobile non documentés. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="75" customHeight="1" s="48">
+      <c r="B24" s="96" t="n">
+        <v>74</v>
+      </c>
+      <c r="C24" s="95" t="inlineStr">
+        <is>
+          <t>Politique de crédit et de recouvrement du Grenier : règles d'octroi, recouvrement des agents sortis ou non précomptés, traitement des prêts à mécano anormal.</t>
+        </is>
+      </c>
+      <c r="D24" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E24" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F24" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « POLITIK DE CREDIT DU GRENIER VFVF.doc »</t>
+        </is>
+      </c>
+      <c r="G24" s="95" t="inlineStr">
+        <is>
+          <t>Politique de crédit du Grenier. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="75" customHeight="1" s="48">
+      <c r="B25" s="96" t="n">
+        <v>76</v>
+      </c>
+      <c r="C25" s="95" t="inlineStr">
+        <is>
+          <t>Fichier du personnel du FPPN au 31/12/2025 et au 31/08/2026 : date de naissance, date d'embauche, salaire mensuel, catégorie, âge de départ prévu.</t>
+        </is>
+      </c>
+      <c r="D25" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E25" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F25" s="95" t="inlineStr">
+        <is>
+          <t>04-Nouveaux Personnel et paie : « DISA_256927_2021.xls » à « DISA_256927_2025.xls » (colonnes ANNEE NAISS., DATE EMBAUCHE, DATE DEPART, SALAIRE BRUT)</t>
+        </is>
+      </c>
+      <c r="G25" s="95" t="inlineStr">
+        <is>
+          <t>Les DISA donnent, pour chaque salarié déclaré à la CNPS, l'année de naissance, la date d'embauche et le salaire brut annuel : base possible de la provision pour départ à la retraite. Situation au 31/08/2026 non reçue. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="75" customHeight="1" s="48">
+      <c r="B26" s="96" t="n">
+        <v>80</v>
+      </c>
+      <c r="C26" s="95" t="inlineStr">
+        <is>
+          <t>Conventions, taux, échéances et relevés du DAT BOA (compte 52210200) de 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="D26" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E26" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F26" s="95" t="inlineStr">
+        <is>
+          <t>07-Nouveaux Trésorerie et placements : états de rapprochement bancaire 2020 à 2026</t>
+        </is>
+      </c>
+      <c r="G26" s="95" t="inlineStr">
+        <is>
+          <t>Mouvements des comptes BOA à lire ; conventions et relevés du DAT non reçus. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="75" customHeight="1" s="48">
+      <c r="B27" s="96" t="n">
+        <v>83</v>
+      </c>
+      <c r="C27" s="95" t="inlineStr">
+        <is>
+          <t>Correspondance avec Orabank sur l'arrêt des prélèvements mensuels et le remboursement du DAT.</t>
+        </is>
+      </c>
+      <c r="D27" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E27" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F27" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf »</t>
+        </is>
+      </c>
+      <c r="G27" s="95" t="inlineStr">
+        <is>
+          <t>La convention doit préciser la dénomination et le statut de la structure CMP. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="75" customHeight="1" s="48">
+      <c r="B28" s="96" t="n">
+        <v>84</v>
+      </c>
+      <c r="C28" s="95" t="inlineStr">
+        <is>
+          <t>Titres de propriété ou actes d'acquisition des terrains, situation de chaque terrain (projet, attribution, litige).</t>
+        </is>
+      </c>
+      <c r="D28" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E28" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F28" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « Certificat de Propriété Terrain Marcori (Siège).pdf » ; « Certificat de Propriété Terrain Plateau.pdf » ; « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE… »</t>
+        </is>
+      </c>
+      <c r="G28" s="95" t="inlineStr">
+        <is>
+          <t>Deux certificats de propriété et un acte de vente reçus ; situation de chaque terrain (projet, attribution, litige) non reçue. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="75" customHeight="1" s="48">
+      <c r="B29" s="96" t="n">
+        <v>88</v>
+      </c>
+      <c r="C29" s="95" t="inlineStr">
+        <is>
+          <t>Bilan d'ouverture de la clinique du FPPN (CMP) et détail des comptes 47111104 et 47111105.</t>
+        </is>
+      </c>
+      <c r="D29" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E29" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F29" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf » (scan)</t>
+        </is>
+      </c>
+      <c r="G29" s="95" t="inlineStr">
+        <is>
+          <t>Convention de la clinique (CMP) avec Transvie reçue ; bilan d'ouverture et détail des comptes 47111104 et 47111105 non reçus. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="75" customHeight="1" s="48">
+      <c r="B30" s="96" t="n">
+        <v>90</v>
+      </c>
+      <c r="C30" s="95" t="inlineStr">
+        <is>
+          <t>Liste des comptes bancaires, actifs et inactifs, avec leurs signataires.</t>
+        </is>
+      </c>
+      <c r="D30" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E30" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F30" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « LISTE DES COMPTES BANCAIRES  DU FPPN.pdf » ; « Habilitation de signatures.pdf » (scans)</t>
+        </is>
+      </c>
+      <c r="G30" s="95" t="inlineStr">
+        <is>
+          <t>Liste des comptes bancaires et habilitations de signature. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="75" customHeight="1" s="48">
+      <c r="B31" s="96" t="n">
+        <v>93</v>
+      </c>
+      <c r="C31" s="95" t="inlineStr">
+        <is>
+          <t>Barème officiel des allocations décès par grade (sous-officier, officier, commissaire).</t>
+        </is>
+      </c>
+      <c r="D31" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E31" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F31" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf »</t>
+        </is>
+      </c>
+      <c r="G31" s="95" t="inlineStr">
+        <is>
+          <t>Barème des allocations décès par grade à lire dans le cahier des charges 2021. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="75" customHeight="1" s="48">
+      <c r="B32" s="96" t="n">
+        <v>97</v>
+      </c>
+      <c r="C32" s="95" t="inlineStr">
+        <is>
+          <t>Déclarations CNPS de 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="D32" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E32" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F32" s="95" t="inlineStr">
+        <is>
+          <t>04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025</t>
+        </is>
+      </c>
+      <c r="G32" s="95" t="inlineStr">
+        <is>
+          <t>DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="75" customHeight="1" s="48">
+      <c r="B33" s="96" t="n">
+        <v>99</v>
+      </c>
+      <c r="C33" s="95" t="inlineStr">
+        <is>
+          <t>Décision fixant le taux servi de 3,5 % sur le PEP et l'EFC.</t>
+        </is>
+      </c>
+      <c r="D33" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E33" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F33" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : manuel de produit d'épargne ; cahier des charges EFC et PEP 2021</t>
+        </is>
+      </c>
+      <c r="G33" s="95" t="inlineStr">
+        <is>
+          <t>Taux servi de 3,5 % à vérifier dans ces documents ; décision non reçue. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="75" customHeight="1" s="48">
+      <c r="B34" s="96" t="n">
+        <v>100</v>
+      </c>
+      <c r="C34" s="95" t="inlineStr">
+        <is>
+          <t>Cahier des charges du régime des prestations sociales du FPPN en vigueur, et versions applicables depuis 2020 (cité aux articles 21 et 40 à 42 du règlement inté</t>
+        </is>
+      </c>
+      <c r="D34" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E34" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F34" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (17 p.) ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » (10 p.)</t>
+        </is>
+      </c>
+      <c r="G34" s="95" t="inlineStr">
+        <is>
+          <t>Cahiers des charges du régime des prestations sociales, version 2021. Versions antérieures à 2021 non reçues. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="75" customHeight="1" s="48">
+      <c r="B35" s="96" t="n">
+        <v>101</v>
+      </c>
+      <c r="C35" s="95" t="inlineStr">
+        <is>
+          <t>Tableau des allocations en vigueur de 2020 au 31/08/2026 : allocation décès du membre, allocation décès des ayants droit, allocation d'invalidité par corps (art</t>
+        </is>
+      </c>
+      <c r="D35" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E35" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F35" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf »</t>
+        </is>
+      </c>
+      <c r="G35" s="95" t="inlineStr">
+        <is>
+          <t>Le tableau des allocations doit figurer dans le cahier des charges 2021 ; versions 2020 et postérieures à vérifier. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="75" customHeight="1" s="48">
+      <c r="B36" s="96" t="n">
+        <v>102</v>
+      </c>
+      <c r="C36" s="95" t="inlineStr">
+        <is>
+          <t>Manuels de procédure du Plan Epargne Plus et de l'Entraide de Fin de Carrière : prestations, rémunération servie, conditions de sortie et de rachat (articles 69</t>
+        </is>
+      </c>
+      <c r="D36" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E36" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F36" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »</t>
+        </is>
+      </c>
+      <c r="G36" s="95" t="inlineStr">
+        <is>
+          <t>Manuel des produits d'épargne (PEP et EFC). Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="75" customHeight="1" s="48">
+      <c r="B37" s="96" t="n">
+        <v>103</v>
+      </c>
+      <c r="C37" s="95" t="inlineStr">
+        <is>
+          <t>Fichier du personnel de la Direction Générale avec une colonne de statut : personnel civil salarié ou fonctionnaire de police en service (article 31 du règlemen</t>
+        </is>
+      </c>
+      <c r="D37" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E37" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F37" s="95" t="inlineStr">
+        <is>
+          <t>04-Nouveaux Personnel et paie : DISA 2021 à 2025 ; « RECAPSALAIRES » des états 301</t>
+        </is>
+      </c>
+      <c r="G37" s="95" t="inlineStr">
+        <is>
+          <t>Les DISA couvrent les salariés déclarés à la CNPS (personnel civil) ; les fonctionnaires de police en service n'y figurent a priori pas. Statut à confirmer. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="75" customHeight="1" s="48">
+      <c r="B38" s="96" t="n">
+        <v>107</v>
+      </c>
+      <c r="C38" s="95" t="inlineStr">
+        <is>
+          <t>Procès-verbaux des Assemblées Générales d'affectation des résultats de 2020 à 2025 (article 90 des statuts : réserve légale de 20 % à 50 % de l'excédent net).</t>
+        </is>
+      </c>
+      <c r="D38" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E38" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F38" s="95" t="inlineStr">
+        <is>
+          <t>03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan)</t>
+        </is>
+      </c>
+      <c r="G38" s="95" t="inlineStr">
+        <is>
+          <t>PV de l'AG ordinaire du 15/02/2024 reçu ; autres AG d'affectation non reçues. Contenu à analyser.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:G3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
PBC : pointage du contenu du lot 1 (21 items, 5 points) et préparation du lot 2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261022.xlsx
+++ b/FPPN_PBC_complete_pointee_20261022.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Points à clarifier" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage autres équipes" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage nouveaux fichiers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage lot 1 (contenu)" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PBC Actuariat FPPN'!$B$12:$P$12</definedName>
@@ -24,9 +25,10 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Synthèse du pointage'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Détail par mois'!$B$5:$E$1605</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Points à clarifier'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Points à clarifier'!$A$1:$E$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Points à clarifier'!$A$1:$E$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pointage autres équipes'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Pointage nouveaux fichiers'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Pointage lot 1 (contenu)'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -1088,7 +1090,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="192" customHeight="1" s="48">
+    <row r="12" ht="267" customHeight="1" s="48">
       <c r="B12" s="70">
         <f>+B11+1</f>
         <v/>
@@ -1117,7 +1119,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026. Seuls des fichiers de précomptes ont été reçus : ils ne décrivent pas les prestations.
 Pointage des autres équipes (22/10/2026) : Document intitulé « cartographie des risques » contenant les barèmes des prestations, reçu par l'équipe comptable le 20/10/2026. Copie à obtenir auprès de l'équipe d'audit comptable. Cahier des charges (item 100) toujours attendu.
-Nouveaux fichiers du 22/10/2026 : Règles et barèmes des prestations (maladie, invalidité-décès, EFC, PEP). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ».</t>
+Nouveaux fichiers du 22/10/2026 : Règles et barèmes des prestations (maladie, invalidité-décès, EFC, PEP). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ».
+Lot 1 lu le 22/10/2026 : Lu : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf », « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » et « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » (maternité : 3 échographies, 3 consultations, allocation d'accouchement de 100 000 FCFA).</t>
         </is>
       </c>
       <c r="M12" s="76" t="inlineStr">
@@ -1282,7 +1285,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="147" customHeight="1" s="48">
+    <row r="19" ht="207" customHeight="1" s="48">
       <c r="B19" s="70">
         <f>+B18+1</f>
         <v/>
@@ -1311,7 +1314,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Rapports actuariels et calcul des provisions : en attente pour l'équipe comptable également.
-Nouveaux fichiers du 22/10/2026 : Études techniques internes reçues ; aucun rapport actuariel ni calcul des provisions. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » ; « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » (.docx, .pdf).</t>
+Nouveaux fichiers du 22/10/2026 : Études techniques internes reçues ; aucun rapport actuariel ni calcul des provisions. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » ; « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » (.docx, .pdf).
+Lot 1 lu le 22/10/2026 : Études internes reçues (« ETUDE DES RATIO MALADIE DECES 2.xlsx », « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE », « INTERPRETATION DES RATIOS… ») ; aucun rapport actuariel ni calcul des provisions.</t>
         </is>
       </c>
       <c r="M19" s="76" t="inlineStr">
@@ -1662,7 +1666,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="102" customHeight="1" s="48">
+    <row r="34" ht="147" customHeight="1" s="48">
       <c r="B34" s="70">
         <f>+B31+1</f>
         <v/>
@@ -1690,7 +1694,8 @@
       <c r="K34" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026. Les fichiers de versements EFC 870 et PEP 998 reçus ne décrivent pas les règles des produits.
-Nouveaux fichiers du 22/10/2026 : Description des produits d'épargne EFC et PEP. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Description des produits d'épargne EFC et PEP. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ».
+Lot 1 lu le 22/10/2026 : Lu : « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » et « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ». Taux servis contradictoires : voir le point à clarifier sur l'EFC.</t>
         </is>
       </c>
       <c r="M34" s="76" t="inlineStr">
@@ -1739,7 +1744,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="102" customHeight="1" s="48">
+    <row r="36" ht="222" customHeight="1" s="48">
       <c r="B36" s="70">
         <f>+B35+1</f>
         <v/>
@@ -1767,7 +1772,8 @@
       <c r="K36" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Nouveaux fichiers du 22/10/2026 : Taux crédité à rechercher dans le manuel et le cahier des charges ; décisions annuelles non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; cahier des charges EFC et PEP 2021.</t>
+Nouveaux fichiers du 22/10/2026 : Taux crédité à rechercher dans le manuel et le cahier des charges ; décisions annuelles non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; cahier des charges EFC et PEP 2021.
+Lot 1 lu le 22/10/2026 : Trois taux écrits pour l'EFC : 5,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » et « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx », « à partir de 2024 »), intérêt simple de 14 % au-delà de 2024 et pour les souscriptions postérieures au cahier des charges (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf »), 3,5 % selon le chef comptable (19/10/2026). PEP : 3,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »). Décision fixant le taux appliqué chaque année non reçue.</t>
         </is>
       </c>
       <c r="M36" s="76" t="inlineStr">
@@ -1825,7 +1831,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="162" customHeight="1" s="48">
+    <row r="40" ht="222" customHeight="1" s="48">
       <c r="B40" s="70">
         <f>+B37+1</f>
         <v/>
@@ -1858,7 +1864,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : État des placements, dossiers des DAT et tableau de synthèse en attente pour l'équipe comptable également.
-Nouveaux fichiers du 22/10/2026 : États de rapprochement bancaire 2020 à 2026 reçus ; échéancier des placements (DAT, FCP) non reçu. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » (onglets par banque : BOA PEP, BOA EFC, BOA BF, BOA FPPN, ORABANK, BANQUE ATLANTIQUE).</t>
+Nouveaux fichiers du 22/10/2026 : États de rapprochement bancaire 2020 à 2026 reçus ; échéancier des placements (DAT, FCP) non reçu. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » (onglets par banque : BOA PEP, BOA EFC, BOA BF, BOA FPPN, ORABANK, BANQUE ATLANTIQUE).
+Lot 1 lu le 22/10/2026 : Lu : « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » : solde bancaire et solde comptable mensuels par compte (BOA EFC, BOA PEP, BOA BF, BOA FPPN, Orabank, Banque Atlantique). Échéancier des placements (DAT, FCP) non reçu.</t>
         </is>
       </c>
       <c r="M40" s="76" t="inlineStr">
@@ -2105,7 +2112,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="117" customHeight="1" s="48">
+    <row r="51" ht="192" customHeight="1" s="48">
       <c r="B51" s="70">
         <f>+B48+1</f>
         <v/>
@@ -2137,7 +2144,8 @@
       <c r="K51" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Nouveaux fichiers du 22/10/2026 : Sinistralité observée par le FPPN (au 30 juin, historique 2015 à 2021) et interprétation : méthode du FPPN à confronter à la formule de la Décision n° 05/2022. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » (onglets Tableau, Notes, Historique 2015-2021) ; « INTERPRETATION DES RATIOS… » (.docx, .pdf).</t>
+Nouveaux fichiers du 22/10/2026 : Sinistralité observée par le FPPN (au 30 juin, historique 2015 à 2021) et interprétation : méthode du FPPN à confronter à la formule de la Décision n° 05/2022. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » (onglets Tableau, Notes, Historique 2015-2021) ; « INTERPRETATION DES RATIOS… » (.docx, .pdf).
+Lot 1 lu le 22/10/2026 : Lu : « ETUDE DES RATIO MALADIE DECES 2.xlsx » : cotisations et sinistres décès, nombre d'adhérents et de décès (adhérents, conjoints, enfants) de 2015 au 30/06/2026 ; notes de calcul de la sinistralité décès (13 %) et maladie (99,23 %) au 30/06/2026. Détail mensuel maladie non reçu.</t>
         </is>
       </c>
       <c r="M51" s="76" t="inlineStr">
@@ -2226,7 +2234,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="147" customFormat="1" customHeight="1" s="68">
+    <row r="54" ht="192" customFormat="1" customHeight="1" s="68">
       <c r="B54" s="70">
         <f>+B53+1</f>
         <v/>
@@ -2255,7 +2263,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Barèmes en vigueur reçus dans la « cartographie des risques » (20/10/2026). Barèmes successifs depuis 2001 et décisions non reçus. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : Barèmes 2021 reçus ; barèmes successifs depuis 2001 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : cartographie des risques.</t>
+Nouveaux fichiers du 22/10/2026 : Barèmes 2021 reçus ; barèmes successifs depuis 2001 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : cahiers des charges 2021 ; 05-Nouveaux Prestations : cartographie des risques.
+Lot 1 lu le 22/10/2026 : Barèmes 2021 à 2026 reçus (« CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ») ; barèmes successifs de 2001 à 2020 et décisions non reçus.</t>
         </is>
       </c>
       <c r="M54" s="76" t="inlineStr">
@@ -2336,7 +2345,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="147" customHeight="1" s="48">
+    <row r="57" ht="192" customHeight="1" s="48">
       <c r="B57" s="70">
         <f>+B56+1</f>
         <v/>
@@ -2365,7 +2374,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Liste des pièces du dossier d'allocation décès et conditions d'octroi en attente (M. Soumahoro).
-Nouveaux fichiers du 22/10/2026 : Listes des pièces exigées pour les prestations décès ; cahier des charges reçu (item 100). Fichiers : 05-Nouveaux Prestations : « Liste des pièces à fournir en cas de décès d'un membre participant.pdf », « … d'un ayant-droit.pdf », « … pour les frais funeraires.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Listes des pièces exigées pour les prestations décès ; cahier des charges reçu (item 100). Fichiers : 05-Nouveaux Prestations : « Liste des pièces à fournir en cas de décès d'un membre participant.pdf », « … d'un ayant-droit.pdf », « … pour les frais funeraires.pdf ».
+Lot 1 lu le 22/10/2026 : Lu : trois listes de pièces (décès d'un membre, d'un ayant droit, frais funéraires) et pièces exigées dans « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».</t>
         </is>
       </c>
       <c r="M57" s="76" t="inlineStr">
@@ -2834,7 +2844,7 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="102" customHeight="1" s="48">
+    <row r="74" ht="177" customHeight="1" s="48">
       <c r="B74" s="70">
         <f>+B73+1</f>
         <v/>
@@ -2862,7 +2872,8 @@
       <c r="K74" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
-Nouveaux fichiers du 22/10/2026 : Règlement du PEP et de l'EFC. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Règlement du PEP et de l'EFC. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ».
+Lot 1 lu le 22/10/2026 : Lu : PEP 1 à 3 (10 000 à 50 000 FCFA et plus, durée de 3 à 11 ans, rachats partiels limités à deux, pénalité de 10 %, rupture anticipée pénalisée de 14 %) ; EFC 1 à 3 (6 000 ou 10 000 FCFA par mois jusqu'à la retraite, retrait seulement en fin de carrière).</t>
         </is>
       </c>
       <c r="M74" s="76" t="inlineStr">
@@ -3238,7 +3249,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="102" customHeight="1" s="48">
+    <row r="87" ht="177" customHeight="1" s="48">
       <c r="B87" s="70">
         <f>+B86+1</f>
         <v/>
@@ -3270,7 +3281,8 @@
       <c r="K87" s="75" t="inlineStr">
         <is>
           <t>Demande issue de l'entretien du 19/10/2026 avec le responsable des cotisations (PBC complémentaire cotisations).
-Nouveaux fichiers du 22/10/2026 : EFC, PEP et Grenier documentés ; MEDOC et flotte automobile non documentés. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne, cahiers des charges 2021, « POLITIK DE CREDIT DU GRENIER VFVF.doc ».</t>
+Nouveaux fichiers du 22/10/2026 : EFC, PEP et Grenier documentés ; MEDOC et flotte automobile non documentés. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne, cahiers des charges 2021, « POLITIK DE CREDIT DU GRENIER VFVF.doc ».
+Lot 1 lu le 22/10/2026 : EFC, PEP (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf », « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »), Grenier (« POLITIK DE CREDIT DU GRENIER VFVF.doc ») et flotte automobile (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx », chapitre II) documentés ; MEDOC non documenté.</t>
         </is>
       </c>
       <c r="M87" s="76" t="inlineStr">
@@ -3884,7 +3896,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="147" customHeight="1" s="48">
+    <row r="106" ht="192" customHeight="1" s="48">
       <c r="B106" s="70">
         <f>+B105+1</f>
         <v/>
@@ -3913,7 +3925,8 @@
         <is>
           <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
 Pointage des autres équipes (22/10/2026) : Règlement des crédits reçu ; aucune politique écrite de dépréciation (le FPPN cite les garanties et un taux de 1 %). Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : Politique de crédit du Grenier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « POLITIK DE CREDIT DU GRENIER VFVF.doc ».</t>
+Nouveaux fichiers du 22/10/2026 : Politique de crédit du Grenier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « POLITIK DE CREDIT DU GRENIER VFVF.doc ».
+Lot 1 lu le 22/10/2026 : Reçu : « POLITIK DE CREDIT DU GRENIER VFVF.doc » (environ 98 000 caractères) ; lecture détaillée à faire pour la dépréciation des prêts.</t>
         </is>
       </c>
       <c r="M106" s="76" t="inlineStr">
@@ -3960,7 +3973,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="177" customHeight="1" s="48">
+    <row r="108" ht="267" customHeight="1" s="48">
       <c r="B108" s="70">
         <f>+B107+1</f>
         <v/>
@@ -3993,7 +4006,8 @@
         <is>
           <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
 Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi).
-Nouveaux fichiers du 22/10/2026 : Les DISA donnent, pour chaque salarié déclaré à la CNPS, l'année de naissance, la date d'embauche et le salaire brut annuel : base possible de la provision pour départ à la retraite. Situation au 31/08/2026 non reçue. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « DISA_256927_2021.xls » à « DISA_256927_2025.xls » (colonnes ANNEE NAISS., DATE EMBAUCHE, DATE DEPART, SALAIRE BRUT).</t>
+Nouveaux fichiers du 22/10/2026 : Les DISA donnent, pour chaque salarié déclaré à la CNPS, l'année de naissance, la date d'embauche et le salaire brut annuel : base possible de la provision pour départ à la retraite. Situation au 31/08/2026 non reçue. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « DISA_256927_2021.xls » à « DISA_256927_2025.xls » (colonnes ANNEE NAISS., DATE EMBAUCHE, DATE DEPART, SALAIRE BRUT).
+Lot 1 lu le 22/10/2026 : Lu : « DISA_256927_2021.xls » à « DISA_256927_2025.xls » (DISA 2024 dans « ETAT 301 &amp; DISA 2024 FPPN.xls ») : nom, année de naissance, date d'embauche, salaire brut annuel, durée d'activité par salarié déclaré à la CNPS (80 lignes en 2025). Pas de sexe, de catégorie ni d'âge de départ ; une ligne agrégée « travailleurs occasionnels » ; situation au 31/08/2026 non reçue.</t>
         </is>
       </c>
       <c r="M108" s="76" t="inlineStr">
@@ -4115,7 +4129,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="132" customHeight="1" s="48">
+    <row r="114" ht="177" customHeight="1" s="48">
       <c r="B114" s="70">
         <f>+B111+1</f>
         <v/>
@@ -4148,7 +4162,8 @@
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : Dossiers des DAT en attente pour l'équipe comptable également.
-Nouveaux fichiers du 22/10/2026 : Mouvements des comptes BOA à lire ; conventions et relevés du DAT non reçus. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : états de rapprochement bancaire 2020 à 2026.</t>
+Nouveaux fichiers du 22/10/2026 : Mouvements des comptes BOA à lire ; conventions et relevés du DAT non reçus. Contenu à analyser. Fichiers : 07-Nouveaux Trésorerie et placements : états de rapprochement bancaire 2020 à 2026.
+Lot 1 lu le 22/10/2026 : Mouvements mensuels des comptes BOA lisibles dans « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » ; conventions, taux et relevés du DAT non reçus.</t>
         </is>
       </c>
       <c r="M114" s="76" t="inlineStr">
@@ -4529,7 +4544,7 @@
         </is>
       </c>
     </row>
-    <row r="125" ht="42" customHeight="1" s="48">
+    <row r="125" ht="102" customHeight="1" s="48">
       <c r="B125" s="70">
         <f>+B124+1</f>
         <v/>
@@ -4550,7 +4565,9 @@
       <c r="H125" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I125" s="73" t="n"/>
+      <c r="I125" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J125" s="74" t="inlineStr">
         <is>
           <t>Electronique</t>
@@ -4558,12 +4575,13 @@
       </c>
       <c r="K125" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Lot 1 lu le 22/10/2026 : Les rapprochements bancaires listent des chèques en suspens, dont certains émis depuis décembre 2021 sur le compte BOA EFC et encore non débités au 31/12/2025 (« ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx »).</t>
         </is>
       </c>
       <c r="M125" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4633,7 @@
         </is>
       </c>
     </row>
-    <row r="129" ht="162" customHeight="1" s="48">
+    <row r="129" ht="222" customHeight="1" s="48">
       <c r="B129" s="70">
         <f>+B128+1</f>
         <v/>
@@ -4637,19 +4655,20 @@
         <v>46321</v>
       </c>
       <c r="I129" s="73" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="J129" s="74" t="n"/>
       <c r="K129" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : Barèmes des prestations reçus dans la « cartographie des risques » (20/10/2026), à confronter au barème par grade demandé. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : Barème des allocations décès par grade à lire dans le cahier des charges 2021. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Barème des allocations décès par grade à lire dans le cahier des charges 2021. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».
+Lot 1 lu le 22/10/2026 : Lu : barème par grade dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » ; mêmes montants appliqués dans les notes de « ETUDE DES RATIO MALADIE DECES 2.xlsx » (32 décès au 30/06/2026).</t>
         </is>
       </c>
       <c r="M129" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
+          <t>Reçu</t>
         </is>
       </c>
     </row>
@@ -4756,7 +4775,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="162" customHeight="1" s="48">
+    <row r="133" ht="207" customHeight="1" s="48">
       <c r="B133" s="70">
         <f>+B132+1</f>
         <v/>
@@ -4789,7 +4808,8 @@
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : DISA et état 301 reçus sauf 2026 ; ITS et FDFP reçus (2021 manquant) ; déclarations CNPS en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025.</t>
+Nouveaux fichiers du 22/10/2026 : DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025.
+Lot 1 lu le 22/10/2026 : Lu : états 301 et DISA 2020 à 2025, appels CNPS annuels, DASC 2022, 2023, 2025, fichiers e-CNPS complémentaires 2022. Déclarations mensuelles CNPS et 2026 non reçues.</t>
         </is>
       </c>
       <c r="M133" s="76" t="inlineStr">
@@ -4837,7 +4857,7 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="102" customHeight="1" s="48">
+    <row r="135" ht="147" customHeight="1" s="48">
       <c r="B135" s="70">
         <f>+B134+1</f>
         <v/>
@@ -4865,7 +4885,8 @@
       <c r="K135" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Nouveaux fichiers du 22/10/2026 : Taux servi de 3,5 % à vérifier dans ces documents ; décision non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne ; cahier des charges EFC et PEP 2021.</t>
+Nouveaux fichiers du 22/10/2026 : Taux servi de 3,5 % à vérifier dans ces documents ; décision non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : manuel de produit d'épargne ; cahier des charges EFC et PEP 2021.
+Lot 1 lu le 22/10/2026 : Le taux de 3,5 % n'est écrit que pour le PEP (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ») ; pour l'EFC, les textes donnent 5,5 % ou 14 % simple. Décision non reçue.</t>
         </is>
       </c>
       <c r="M135" s="76" t="inlineStr">
@@ -4882,7 +4903,7 @@
         </is>
       </c>
     </row>
-    <row r="138" ht="117" customHeight="1" s="48">
+    <row r="138" ht="222" customHeight="1" s="48">
       <c r="B138" s="70">
         <f>+B135+1</f>
         <v/>
@@ -4914,7 +4935,8 @@
       <c r="K138" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Nouveaux fichiers du 22/10/2026 : Cahiers des charges du régime des prestations sociales, version 2021. Versions antérieures à 2021 non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (17 p.) ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » (10 p.).</t>
+Nouveaux fichiers du 22/10/2026 : Cahiers des charges du régime des prestations sociales, version 2021. Versions antérieures à 2021 non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (17 p.) ; « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » (10 p.).
+Lot 1 lu le 22/10/2026 : Lu : cahiers des charges 2021 « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (risques couverts, ticket modérateur 80 % / 20 %, exclusions, forclusions, procédures) et « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ». Le tableau des allocations n'y figure pas (renvoi) : il est dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ». Versions antérieures à 2021 non reçues.</t>
         </is>
       </c>
       <c r="M138" s="76" t="inlineStr">
@@ -4923,7 +4945,7 @@
         </is>
       </c>
     </row>
-    <row r="139" ht="162" customHeight="1" s="48">
+    <row r="139" ht="267" customHeight="1" s="48">
       <c r="B139" s="70">
         <f>+B138+1</f>
         <v/>
@@ -4945,7 +4967,7 @@
         <v>46321</v>
       </c>
       <c r="I139" s="73" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="J139" s="74" t="inlineStr">
         <is>
@@ -4956,16 +4978,17 @@
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : Barèmes des prestations reçus dans la « cartographie des risques » (20/10/2026) ; tableau des allocations officiel non identifié. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : Le tableau des allocations doit figurer dans le cahier des charges 2021 ; versions 2020 et postérieures à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Le tableau des allocations doit figurer dans le cahier des charges 2021 ; versions 2020 et postérieures à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».
+Lot 1 lu le 22/10/2026 : Lu : « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » donne les allocations décès par grade (commissaire 2 200 000, officier 1 600 000, sous-officier 1 400 000 FCFA ; conjoint 1 000 000 / 700 000 / 600 000 ; enfant 230 000 / 150 000 / 120 000), pour 2021 à 2023 et 2023 à 2026, avec des frais funéraires de 300 000 FCFA pour le membre sur 2023 à 2026. Allocation d'invalidité non chiffrée.</t>
         </is>
       </c>
       <c r="M139" s="76" t="inlineStr">
         <is>
-          <t>Partiellement Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="132" customHeight="1" s="48">
+          <t>Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="192" customHeight="1" s="48">
       <c r="B140" s="70">
         <f>+B139+1</f>
         <v/>
@@ -4998,7 +5021,8 @@
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : À rechercher dans les manuels de procédures non signés reçus par l'équipe comptable le 21/10/2026.
-Nouveaux fichiers du 22/10/2026 : Manuel des produits d'épargne (PEP et EFC). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ».</t>
+Nouveaux fichiers du 22/10/2026 : Manuel des produits d'épargne (PEP et EFC). Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ».
+Lot 1 lu le 22/10/2026 : Lu : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » (version 2021, certificat d'adoption non daté ni signé) : PEP rémunéré à 3,5 % par an, EFC à 5,5 % par an, intérêts non capitalisés et versés sur le compte courant.</t>
         </is>
       </c>
       <c r="M140" s="76" t="inlineStr">
@@ -5015,7 +5039,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="162" customHeight="1" s="48">
+    <row r="143" ht="237" customHeight="1" s="48">
       <c r="B143" s="70">
         <f>+B140+1</f>
         <v/>
@@ -5048,7 +5072,8 @@
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi) : le statut civil ou policier devra y figurer.
-Nouveaux fichiers du 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS (personnel civil) ; les fonctionnaires de police en service n'y figurent a priori pas. Statut à confirmer. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : DISA 2021 à 2025 ; « RECAPSALAIRES » des états 301.</t>
+Nouveaux fichiers du 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS (personnel civil) ; les fonctionnaires de police en service n'y figurent a priori pas. Statut à confirmer. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : DISA 2021 à 2025 ; « RECAPSALAIRES » des états 301.
+Lot 1 lu le 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS. Les états 301 distinguent des onglets « RECAPSALAIRES 2024 CMP » et « RECAPSALAIRES 2025 GRENIER » : Direction Générale, clinique et Grenier sont identifiables par nom. Le statut des policiers en service n'y figure pas.</t>
         </is>
       </c>
       <c r="M143" s="76" t="inlineStr">
@@ -5391,7 +5416,7 @@
       </c>
       <c r="D6" s="95" t="inlineStr">
         <is>
-          <t>2, 16, 33, 45, 46, 70, 74, 90, 100, 102</t>
+          <t>2, 16, 33, 45, 46, 70, 74, 90, 93, 100, 101, 102</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5432,7 @@
       </c>
       <c r="D7" s="95" t="inlineStr">
         <is>
-          <t>1, 3, 4, 6, 7, 8, 9, 12, 13, 17, 18, 20, 21, 23, 26, 27, 28, 30, 34, 35, 37, 42, 44, 47, 50, 53, 57, 71, 73, 76, 80, 83, 84, 88, 93, 97, 99, 101, 103, 107</t>
+          <t>1, 3, 4, 6, 7, 8, 9, 12, 13, 17, 18, 20, 21, 23, 26, 27, 28, 30, 34, 35, 37, 42, 44, 47, 50, 53, 57, 71, 73, 76, 80, 83, 84, 88, 91, 97, 99, 103, 107</t>
         </is>
       </c>
     </row>
@@ -5423,7 +5448,7 @@
       </c>
       <c r="D8" s="95" t="inlineStr">
         <is>
-          <t>5, 10, 11, 14, 15, 19, 22, 24, 25, 29, 31, 32, 36, 38, 39, 40, 41, 43, 48, 49, 51, 52, 54, 55, 56, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 72, 75, 77, 78, 79, 81, 82, 85, 86, 87, 89, 91, 92, 94, 95, 96, 98, 104, 105, 106, 108, 109</t>
+          <t>5, 10, 11, 14, 15, 19, 22, 24, 25, 29, 31, 32, 36, 38, 39, 40, 41, 43, 48, 49, 51, 52, 54, 55, 56, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 72, 75, 77, 78, 79, 81, 82, 85, 86, 87, 89, 92, 94, 95, 96, 98, 104, 105, 106, 108, 109</t>
         </is>
       </c>
     </row>
@@ -42709,7 +42734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E46"/>
+  <dimension ref="B2:E51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2" customWidth="1" style="77" min="1" max="1"/>
@@ -43571,6 +43596,106 @@
       <c r="E46" s="95" t="inlineStr">
         <is>
           <t>Transmettre les deux documents (items 100 et 101).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="102" customHeight="1" s="48">
+      <c r="B47" s="96" t="n">
+        <v>42</v>
+      </c>
+      <c r="C47" s="95" t="inlineStr">
+        <is>
+          <t>Taux servi sur l'EFC</t>
+        </is>
+      </c>
+      <c r="D47" s="95" t="inlineStr">
+        <is>
+          <t>Trois taux écrits : 5,5 % par an (manuel d'épargne 2021, cartographie), intérêt simple de 14 % (cahier des charges EFC et PEP 2021, au-delà de 2024 et pour les nouvelles souscriptions), 3,5 % (chef comptable). Bonus de 300 000 FCFA cité par le cahier des charges.</t>
+        </is>
+      </c>
+      <c r="E47" s="95" t="inlineStr">
+        <is>
+          <t>Indiquer le taux appliqué chaque année de 2020 à 2026, la décision qui le fixe et le calcul du capital EFC servi à la retraite (items 18 et 99).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="60" customHeight="1" s="48">
+      <c r="B48" s="96" t="n">
+        <v>43</v>
+      </c>
+      <c r="C48" s="95" t="inlineStr">
+        <is>
+          <t>Manuel d'épargne</t>
+        </is>
+      </c>
+      <c r="D48" s="95" t="inlineStr">
+        <is>
+          <t>Le certificat d'adoption du manuel des produits d'épargne (2021) n'est ni daté ni signé.</t>
+        </is>
+      </c>
+      <c r="E48" s="95" t="inlineStr">
+        <is>
+          <t>Transmettre la délibération d'adoption.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="87" customHeight="1" s="48">
+      <c r="B49" s="96" t="n">
+        <v>44</v>
+      </c>
+      <c r="C49" s="95" t="inlineStr">
+        <is>
+          <t>Ayants droit</t>
+        </is>
+      </c>
+      <c r="D49" s="95" t="inlineStr">
+        <is>
+          <t>Règlement intérieur (art. 40) : enfants de 0 à 18 ans, cinq au plus (soins), quatre de 7 à 18 ans (décès). Cahier des charges 2021 : enfants mineurs de moins de 21 ans. Cartographie : six enfants de 5 à 21 ans.</t>
+        </is>
+      </c>
+      <c r="E49" s="95" t="inlineStr">
+        <is>
+          <t>Préciser la règle en vigueur pour les soins et pour les allocations décès.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="72" customHeight="1" s="48">
+      <c r="B50" s="96" t="n">
+        <v>45</v>
+      </c>
+      <c r="C50" s="95" t="inlineStr">
+        <is>
+          <t>Frais funéraires du membre</t>
+        </is>
+      </c>
+      <c r="D50" s="95" t="inlineStr">
+        <is>
+          <t>La cartographie prévoit 300 000 FCFA de frais funéraires pour le membre sur 2023 à 2026 ; l'étude des ratios les applique au 30/06/2026 ; le tableau 2021 à 2023 ne les mentionne pas.</t>
+        </is>
+      </c>
+      <c r="E50" s="95" t="inlineStr">
+        <is>
+          <t>Confirmer la date d'entrée en vigueur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1" s="48">
+      <c r="B51" s="96" t="n">
+        <v>46</v>
+      </c>
+      <c r="C51" s="95" t="inlineStr">
+        <is>
+          <t>Chèques en suspens</t>
+        </is>
+      </c>
+      <c r="D51" s="95" t="inlineStr">
+        <is>
+          <t>Des chèques émis depuis décembre 2021 restent en suspens sur le compte BOA EFC au 31/12/2025.</t>
+        </is>
+      </c>
+      <c r="E51" s="95" t="inlineStr">
+        <is>
+          <t>Expliquer ces chèques et leur traitement (item 91).</t>
         </is>
       </c>
     </row>
@@ -46333,4 +46458,595 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:F26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" style="48" min="2" max="2"/>
+    <col width="48" customWidth="1" style="48" min="3" max="3"/>
+    <col width="16" customWidth="1" style="48" min="4" max="4"/>
+    <col width="16" customWidth="1" style="48" min="5" max="5"/>
+    <col width="100" customWidth="1" style="48" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="97" t="inlineStr">
+        <is>
+          <t>Pointage sur le contenu du lot 1 des nouveaux fichiers (22/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="40" customHeight="1" s="48">
+      <c r="B3" s="79" t="inlineStr">
+        <is>
+          <t>Lot 1 : 61 fichiers reçus, empreintes SHA-256 conformes au journal « journal_lot1.csv ». Chaque statut repose sur la lecture du contenu. Contrôle croisé : les nouvelles balances 2021 et 2025 sont identiques, compte par compte, aux balances déjà exploitées (aucun écart de solde).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="80" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C5" s="80" t="inlineStr">
+        <is>
+          <t>Document demandé (PBC actuarielle)</t>
+        </is>
+      </c>
+      <c r="D5" s="80" t="inlineStr">
+        <is>
+          <t>Statut avant</t>
+        </is>
+      </c>
+      <c r="E5" s="80" t="inlineStr">
+        <is>
+          <t>Statut après</t>
+        </is>
+      </c>
+      <c r="F5" s="80" t="inlineStr">
+        <is>
+          <t>Constat sur le contenu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1" s="48">
+      <c r="B6" s="96" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="95" t="inlineStr">
+        <is>
+          <t>Règlement ou fiche descriptive de chaque prestation servie (allocation décès, invalidité, prise en charge des retraités, santé, épargne, autres aides) : bénéfic</t>
+        </is>
+      </c>
+      <c r="D6" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E6" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F6" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf », « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » et « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » (maternité : 3 échographies, 3 consultations, allocation d'accouchement de 100 000 FCFA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1" s="48">
+      <c r="B7" s="96" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" s="95" t="inlineStr">
+        <is>
+          <t>Tout rapport actuariel, étude technique ou note de calcul des engagements envers les mutualistes existant, quelle que soit sa date.</t>
+        </is>
+      </c>
+      <c r="D7" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E7" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F7" s="95" t="inlineStr">
+        <is>
+          <t>Études internes reçues (« ETUDE DES RATIO MALADIE DECES 2.xlsx », « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE », « INTERPRETATION DES RATIOS… ») ; aucun rapport actuariel ni calcul des provisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1" s="48">
+      <c r="B8" s="96" t="n">
+        <v>16</v>
+      </c>
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>Description des produits d'épargne (épargne de fin de carrière, Plan Épargne Plus, autres) : règles de versement, taux d'intérêt servi ou garanti, conditions de</t>
+        </is>
+      </c>
+      <c r="D8" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E8" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf » et « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ». Taux servis contradictoires : voir le point à clarifier sur l'EFC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" s="48">
+      <c r="B9" s="96" t="n">
+        <v>18</v>
+      </c>
+      <c r="C9" s="95" t="inlineStr">
+        <is>
+          <t>Taux d'intérêt crédité sur l'épargne chaque année et décision qui l'a fixé.</t>
+        </is>
+      </c>
+      <c r="D9" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E9" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F9" s="95" t="inlineStr">
+        <is>
+          <t>Trois taux écrits pour l'EFC : 5,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » et « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx », « à partir de 2024 »), intérêt simple de 14 % au-delà de 2024 et pour les souscriptions postérieures au cahier des charges (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf »), 3,5 % selon le chef comptable (19/10/2026). PEP : 3,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »). Décision fixant le taux appliqué chaque année non reçue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1" s="48">
+      <c r="B10" s="96" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="95" t="inlineStr">
+        <is>
+          <t>Échéancier des placements au 31/12/2025 et au 31/08/2026 : nature, établissement, montant, date de souscription, date d'échéance, taux, conditions de sortie ant</t>
+        </is>
+      </c>
+      <c r="D10" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E10" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F10" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » : solde bancaire et solde comptable mensuels par compte (BOA EFC, BOA PEP, BOA BF, BOA FPPN, Orabank, Banque Atlantique). Échéancier des placements (DAT, FCP) non reçu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1" s="48">
+      <c r="B11" s="96" t="n">
+        <v>27</v>
+      </c>
+      <c r="C11" s="95" t="inlineStr">
+        <is>
+          <t>Fichiers de suivi de la sinistralité de 2019 au 31/08/2026 (tableau de bord du service), avec le détail du calcul du taux de sinistralité.</t>
+        </is>
+      </c>
+      <c r="D11" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E11" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F11" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « ETUDE DES RATIO MALADIE DECES 2.xlsx » : cotisations et sinistres décès, nombre d'adhérents et de décès (adhérents, conjoints, enfants) de 2015 au 30/06/2026 ; notes de calcul de la sinistralité décès (13 %) et maladie (99,23 %) au 30/06/2026. Détail mensuel maladie non reçu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1" s="48">
+      <c r="B12" s="96" t="n">
+        <v>30</v>
+      </c>
+      <c r="C12" s="95" t="inlineStr">
+        <is>
+          <t>Barèmes successifs des capitaux décès, frais funéraires et allocations aux ayants droit, de 2001 à 2026, avec les décisions qui les ont adoptés.</t>
+        </is>
+      </c>
+      <c r="D12" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E12" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F12" s="95" t="inlineStr">
+        <is>
+          <t>Barèmes 2021 à 2026 reçus (« CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ») ; barèmes successifs de 2001 à 2020 et décisions non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1" s="48">
+      <c r="B13" s="96" t="n">
+        <v>33</v>
+      </c>
+      <c r="C13" s="95" t="inlineStr">
+        <is>
+          <t>Liste des pièces exigées pour chaque prestation et cahier du régime des prestations sociales.</t>
+        </is>
+      </c>
+      <c r="D13" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E13" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F13" s="95" t="inlineStr">
+        <is>
+          <t>Lu : trois listes de pièces (décès d'un membre, d'un ayant droit, frais funéraires) et pièces exigées dans « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1" s="48">
+      <c r="B14" s="96" t="n">
+        <v>46</v>
+      </c>
+      <c r="C14" s="95" t="inlineStr">
+        <is>
+          <t>Règlement des produits PEP et EFC : conditions de retrait, échéances, âge de versement, taux servi.</t>
+        </is>
+      </c>
+      <c r="D14" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E14" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F14" s="95" t="inlineStr">
+        <is>
+          <t>Lu : PEP 1 à 3 (10 000 à 50 000 FCFA et plus, durée de 3 à 11 ans, rachats partiels limités à deux, pénalité de 10 %, rupture anticipée pénalisée de 14 %) ; EFC 1 à 3 (6 000 ou 10 000 FCFA par mois jusqu'à la retraite, retrait seulement en fin de carrière).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1" s="48">
+      <c r="B15" s="96" t="n">
+        <v>57</v>
+      </c>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>Documentation de chaque produit : EFC, PEP, MEDOC, prêts du Grenier, flotte automobile (règlement, conditions de souscription, montants, conditions de sortie et</t>
+        </is>
+      </c>
+      <c r="D15" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E15" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F15" s="95" t="inlineStr">
+        <is>
+          <t>EFC, PEP (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf », « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »), Grenier (« POLITIK DE CREDIT DU GRENIER VFVF.doc ») et flotte automobile (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx », chapitre II) documentés ; MEDOC non documenté.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1" s="48">
+      <c r="B16" s="96" t="n">
+        <v>74</v>
+      </c>
+      <c r="C16" s="95" t="inlineStr">
+        <is>
+          <t>Politique de crédit et de recouvrement du Grenier : règles d'octroi, recouvrement des agents sortis ou non précomptés, traitement des prêts à mécano anormal.</t>
+        </is>
+      </c>
+      <c r="D16" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E16" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F16" s="95" t="inlineStr">
+        <is>
+          <t>Reçu : « POLITIK DE CREDIT DU GRENIER VFVF.doc » (environ 98 000 caractères) ; lecture détaillée à faire pour la dépréciation des prêts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1" s="48">
+      <c r="B17" s="96" t="n">
+        <v>76</v>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
+        <is>
+          <t>Fichier du personnel du FPPN au 31/12/2025 et au 31/08/2026 : date de naissance, date d'embauche, salaire mensuel, catégorie, âge de départ prévu.</t>
+        </is>
+      </c>
+      <c r="D17" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E17" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F17" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « DISA_256927_2021.xls » à « DISA_256927_2025.xls » (DISA 2024 dans « ETAT 301 &amp; DISA 2024 FPPN.xls ») : nom, année de naissance, date d'embauche, salaire brut annuel, durée d'activité par salarié déclaré à la CNPS (80 lignes en 2025). Pas de sexe, de catégorie ni d'âge de départ ; une ligne agrégée « travailleurs occasionnels » ; situation au 31/08/2026 non reçue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1" s="48">
+      <c r="B18" s="96" t="n">
+        <v>80</v>
+      </c>
+      <c r="C18" s="95" t="inlineStr">
+        <is>
+          <t>Conventions, taux, échéances et relevés du DAT BOA (compte 52210200) de 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="D18" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E18" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F18" s="95" t="inlineStr">
+        <is>
+          <t>Mouvements mensuels des comptes BOA lisibles dans « ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx » ; conventions, taux et relevés du DAT non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1" s="48">
+      <c r="B19" s="96" t="n">
+        <v>91</v>
+      </c>
+      <c r="C19" s="95" t="inlineStr">
+        <is>
+          <t>État des chèques en suspens et des chèques annulés lors des changements de signataires.</t>
+        </is>
+      </c>
+      <c r="D19" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E19" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F19" s="95" t="inlineStr">
+        <is>
+          <t>Les rapprochements bancaires listent des chèques en suspens, dont certains émis depuis décembre 2021 sur le compte BOA EFC et encore non débités au 31/12/2025 (« ETAT DE RAPPROCHEMENT BANCAIRE FPPN 2020.xlsx » à « … 2026.xlsx »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1" s="48">
+      <c r="B20" s="96" t="n">
+        <v>93</v>
+      </c>
+      <c r="C20" s="95" t="inlineStr">
+        <is>
+          <t>Barème officiel des allocations décès par grade (sous-officier, officier, commissaire).</t>
+        </is>
+      </c>
+      <c r="D20" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E20" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F20" s="95" t="inlineStr">
+        <is>
+          <t>Lu : barème par grade dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » ; mêmes montants appliqués dans les notes de « ETUDE DES RATIO MALADIE DECES 2.xlsx » (32 décès au 30/06/2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1" s="48">
+      <c r="B21" s="96" t="n">
+        <v>97</v>
+      </c>
+      <c r="C21" s="95" t="inlineStr">
+        <is>
+          <t>Déclarations CNPS de 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="D21" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E21" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F21" s="95" t="inlineStr">
+        <is>
+          <t>Lu : états 301 et DISA 2020 à 2025, appels CNPS annuels, DASC 2022, 2023, 2025, fichiers e-CNPS complémentaires 2022. Déclarations mensuelles CNPS et 2026 non reçues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1" s="48">
+      <c r="B22" s="96" t="n">
+        <v>99</v>
+      </c>
+      <c r="C22" s="95" t="inlineStr">
+        <is>
+          <t>Décision fixant le taux servi de 3,5 % sur le PEP et l'EFC.</t>
+        </is>
+      </c>
+      <c r="D22" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E22" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F22" s="95" t="inlineStr">
+        <is>
+          <t>Le taux de 3,5 % n'est écrit que pour le PEP (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx ») ; pour l'EFC, les textes donnent 5,5 % ou 14 % simple. Décision non reçue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1" s="48">
+      <c r="B23" s="96" t="n">
+        <v>100</v>
+      </c>
+      <c r="C23" s="95" t="inlineStr">
+        <is>
+          <t>Cahier des charges du régime des prestations sociales du FPPN en vigueur, et versions applicables depuis 2020 (cité aux articles 21 et 40 à 42 du règlement inté</t>
+        </is>
+      </c>
+      <c r="D23" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E23" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F23" s="95" t="inlineStr">
+        <is>
+          <t>Lu : cahiers des charges 2021 « CAHIER DE CHARGE  MALADIES ET INVAL-DECES 2021.pdf » (risques couverts, ticket modérateur 80 % / 20 %, exclusions, forclusions, procédures) et « CAHIER DE CHARGEEFC &amp; PEP 2021.pdf ». Le tableau des allocations n'y figure pas (renvoi) : il est dans « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx ». Versions antérieures à 2021 non reçues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1" s="48">
+      <c r="B24" s="96" t="n">
+        <v>101</v>
+      </c>
+      <c r="C24" s="95" t="inlineStr">
+        <is>
+          <t>Tableau des allocations en vigueur de 2020 au 31/08/2026 : allocation décès du membre, allocation décès des ayants droit, allocation d'invalidité par corps (art</t>
+        </is>
+      </c>
+      <c r="D24" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E24" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F24" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx » donne les allocations décès par grade (commissaire 2 200 000, officier 1 600 000, sous-officier 1 400 000 FCFA ; conjoint 1 000 000 / 700 000 / 600 000 ; enfant 230 000 / 150 000 / 120 000), pour 2021 à 2023 et 2023 à 2026, avec des frais funéraires de 300 000 FCFA pour le membre sur 2023 à 2026. Allocation d'invalidité non chiffrée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1" s="48">
+      <c r="B25" s="96" t="n">
+        <v>102</v>
+      </c>
+      <c r="C25" s="95" t="inlineStr">
+        <is>
+          <t>Manuels de procédure du Plan Epargne Plus et de l'Entraide de Fin de Carrière : prestations, rémunération servie, conditions de sortie et de rachat (articles 69</t>
+        </is>
+      </c>
+      <c r="D25" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="E25" s="95" t="inlineStr">
+        <is>
+          <t>Reçu</t>
+        </is>
+      </c>
+      <c r="F25" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » (version 2021, certificat d'adoption non daté ni signé) : PEP rémunéré à 3,5 % par an, EFC à 5,5 % par an, intérêts non capitalisés et versés sur le compte courant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1" s="48">
+      <c r="B26" s="96" t="n">
+        <v>103</v>
+      </c>
+      <c r="C26" s="95" t="inlineStr">
+        <is>
+          <t>Fichier du personnel de la Direction Générale avec une colonne de statut : personnel civil salarié ou fonctionnaire de police en service (article 31 du règlemen</t>
+        </is>
+      </c>
+      <c r="D26" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E26" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F26" s="95" t="inlineStr">
+        <is>
+          <t>Les DISA couvrent les salariés déclarés à la CNPS. Les états 301 distinguent des onglets « RECAPSALAIRES 2024 CMP » et « RECAPSALAIRES 2025 GRENIER » : Direction Générale, clinique et Grenier sont identifiables par nom. Le statut des policiers en service n'y figure pas.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rapport v9 : documents du 22/10/2026, périmètre et validité des analyses, provision du personnel recalculée agent par agent ; PBC pointée sur les lots 2 et 3
- validité à trois niveaux (diapositive, ligne « Valable pour », annexe) et colonne dans le classeur
- contrôles croisés : états financiers, effectifs 8Z6, rapport 8Z6 / 936, rapprochements bancaires
- méthode de sinistralité du FPPN, mortalité brute, taux servis sur l'épargne, absence d'intérêts comptabilisés
- PIDR à partir des DISA, séparée DG, CMP, Grenier, avec sensibilités
- PBC : items 110 à 114, 21 items pointés sur le contenu des lots 2 et 3

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_PBC_complete_pointee_20261022.xlsx
+++ b/FPPN_PBC_complete_pointee_20261022.xlsx
@@ -16,19 +16,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage autres équipes" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage nouveaux fichiers" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage lot 1 (contenu)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pointage lots 2 et 3 (contenu)" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PBC Actuariat FPPN'!$B$12:$P$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'PBC Actuariat FPPN'!$1:$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PBC Actuariat FPPN'!$A$1:$N$152</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PBC Actuariat FPPN'!$A$1:$N$158</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Synthèse du pointage'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Synthèse du pointage'!$A$1:$D$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Détail par mois'!$B$5:$E$1605</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Points à clarifier'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Points à clarifier'!$A$1:$E$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Points à clarifier'!$A$1:$E$57</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Pointage autres équipes'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Pointage nouveaux fichiers'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Pointage lot 1 (contenu)'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Pointage lots 2 et 3 (contenu)'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
@@ -943,7 +945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B4:M151"/>
+  <dimension ref="B4:M157"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.18359375" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.82" customWidth="1" style="44" min="1" max="1"/>
@@ -1166,7 +1168,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="252" customHeight="1" s="48">
+    <row r="14" ht="357" customHeight="1" s="48">
       <c r="B14" s="70">
         <f>+B13+1</f>
         <v/>
@@ -1195,7 +1197,8 @@
         <is>
           <t>Convention et avenants : non reçus. Reçu, fichiers de gestion : précomptes retour CGRAE : 30 mois sur 80 (février à mai 2024, juillet 2024 à août 2026) ; manque : janvier 2020 à janvier 2024, juin 2024. Bordereaux : 26 mois sur 80 (février 2024 à septembre 2025, novembre 2025 à janvier 2026, mai à juillet 2026) ; manque : janvier 2020 à janvier 2024, octobre 2025, février à avril 2026, août 2026. Pièces des retraités : 28 mois sur 80 (février 2024 à janvier 2026, mai à août 2026) ; manque : janvier 2020 à janvier 2024, février à avril 2026.
 Pointage des autres équipes (22/10/2026) : Tableau récapitulatif des contrats et conventions (dont CGRAE) reçu partiellement par l'équipe comptable ; liste complète en attente.
-Nouveaux fichiers du 22/10/2026 : Convention avec la CGRAE reçue ; avenants à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan, 9 p.).</t>
+Nouveaux fichiers du 22/10/2026 : Convention avec la CGRAE reçue ; avenants à vérifier. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan, 9 p.).
+Lots 2 et 3 lus le 22/10/2026 : Lu : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan) : précompte sur pension des cotisations de prise en charge médicale (art. 3), pas de suspension des soins pour retard de la CGRAE (art. 4.1 e), précompte dans la limite de la quotité cessible (art. 4.2 a), aucun frais de gestion (art. 5). Annexe 2 (bulletin de souscription) et montant de la cotisation non reçus.</t>
         </is>
       </c>
       <c r="M14" s="76" t="inlineStr">
@@ -1249,7 +1252,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="132" customHeight="1" s="48">
+    <row r="18" ht="192" customHeight="1" s="48">
       <c r="B18" s="70">
         <f>+B15+1</f>
         <v/>
@@ -1276,7 +1279,8 @@
       <c r="J18" s="74" t="n"/>
       <c r="K18" s="75" t="inlineStr">
         <is>
-          <t>Reçu : balances et grands livres (comptes et tiers), aux dates 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025, et 31/08/2026 en impression provisoire. Ils donnent les soldes, pas le détail ni le calcul des provisions. Les balances 2020 donnent les totaux de l'année entière (colonne de cumul au 31/08/2020). Manque : situation au 31/12/2019 ; détail des écritures de janvier à août 2020 ; détail par nature et par garantie et note de calcul, à chacune des 8 dates.</t>
+          <t>Reçu : balances et grands livres (comptes et tiers), aux dates 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025, et 31/08/2026 en impression provisoire. Ils donnent les soldes, pas le détail ni le calcul des provisions. Les balances 2020 donnent les totaux de l'année entière (colonne de cumul au 31/08/2020). Manque : situation au 31/12/2019 ; détail des écritures de janvier à août 2020 ; détail par nature et par garantie et note de calcul, à chacune des 8 dates.
+Lots 2 et 3 lus le 22/10/2026 : Les états financiers 2020 au 31/08/2026 montrent les provisions au passif sans détail par garantie (« ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf » et « ETATS FINANCIERS AU 31-08-2026.pdf »).</t>
         </is>
       </c>
       <c r="M18" s="76" t="inlineStr">
@@ -1285,7 +1289,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="207" customHeight="1" s="48">
+    <row r="19" ht="327" customHeight="1" s="48">
       <c r="B19" s="70">
         <f>+B18+1</f>
         <v/>
@@ -1315,7 +1319,8 @@
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Rapports actuariels et calcul des provisions : en attente pour l'équipe comptable également.
 Nouveaux fichiers du 22/10/2026 : Études techniques internes reçues ; aucun rapport actuariel ni calcul des provisions. Contenu à analyser. Fichiers : 05-Nouveaux Prestations : « ETUDE DES RATIO MALADIE DECES 2.xlsx » ; « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE » (.docx, .pdf).
-Lot 1 lu le 22/10/2026 : Études internes reçues (« ETUDE DES RATIO MALADIE DECES 2.xlsx », « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE », « INTERPRETATION DES RATIOS… ») ; aucun rapport actuariel ni calcul des provisions.</t>
+Lot 1 lu le 22/10/2026 : Études internes reçues (« ETUDE DES RATIO MALADIE DECES 2.xlsx », « RAPPORT GLOBAL SUR LE SERVICE ASSURANCE MALADIE », « INTERPRETATION DES RATIOS… ») ; aucun rapport actuariel ni calcul des provisions.
+Lots 2 et 3 lus le 22/10/2026 : Lus : rapports de gestion et rapports moraux 2020 à 2025 (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf ») : analyses de l'excédent et de l'épargne, sans calcul actuariel des engagements.</t>
         </is>
       </c>
       <c r="M19" s="76" t="inlineStr">
@@ -1487,7 +1492,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="222" customHeight="1" s="48">
+    <row r="26" ht="342" customHeight="1" s="48">
       <c r="B26" s="70">
         <f>+B25+1</f>
         <v/>
@@ -1519,7 +1524,8 @@
       <c r="K26" s="75" t="inlineStr">
         <is>
           <t>Reçu : fichiers aller (envoyés par le FPPN) et retour (précomptes de la Solde ou de la CGRAE), par mutualiste et par mois. Maladie 936 : 31 mois sur 80 (janvier à novembre 2024, janvier 2025 à août 2026) ; illisible : décembre 2024 ; manque : 2020 à 2023. Décès 8Z6 : 24 mois sur 80 (janvier à avril 2024, novembre 2024, janvier à mars 2025, mai 2025 à août 2026) ; illisible : décembre 2024 ; manque : 2020 à 2023, mai à octobre 2024, avril 2025. Retraités CGRAE : 30 mois sur 80 (février à mai 2024, juillet 2024 à août 2026) ; manque : janvier 2020 à janvier 2024, juin 2024. Manque : état des cotisations appelées et encaissées par mois et par catégorie.
-Pointage des autres équipes (22/10/2026) : Précomptes 2020 à 2022 (Easy Money) et état des cotisations de la Solde 2020 à 2023 non reçus ; aucun rapprochement entre fichiers retour et comptabilité (relance 2.2 : non applicable).</t>
+Pointage des autres équipes (22/10/2026) : Précomptes 2020 à 2022 (Easy Money) et état des cotisations de la Solde 2020 à 2023 non reçus ; aucun rapprochement entre fichiers retour et comptabilité (relance 2.2 : non applicable).
+Lots 2 et 3 lus le 22/10/2026 : Les rapports de gestion donnent les cotisations maladie annuelles (« Cotisation Maladie (3,5 % SB) »), sans détail mensuel ni par catégorie (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf »).</t>
         </is>
       </c>
       <c r="M26" s="76" t="inlineStr">
@@ -1744,7 +1750,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="222" customHeight="1" s="48">
+    <row r="36" ht="267" customHeight="1" s="48">
       <c r="B36" s="70">
         <f>+B35+1</f>
         <v/>
@@ -1773,7 +1779,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Nouveaux fichiers du 22/10/2026 : Taux crédité à rechercher dans le manuel et le cahier des charges ; décisions annuelles non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » ; cahier des charges EFC et PEP 2021.
-Lot 1 lu le 22/10/2026 : Trois taux écrits pour l'EFC : 5,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » et « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx », « à partir de 2024 »), intérêt simple de 14 % au-delà de 2024 et pour les souscriptions postérieures au cahier des charges (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf »), 3,5 % selon le chef comptable (19/10/2026). PEP : 3,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »). Décision fixant le taux appliqué chaque année non reçue.</t>
+Lot 1 lu le 22/10/2026 : Trois taux écrits pour l'EFC : 5,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx » et « CARTOGRAPHIE DES RISQUES COUVERTS ET DES PRESTATIONS OFFERTES.docx », « à partir de 2024 »), intérêt simple de 14 % au-delà de 2024 et pour les souscriptions postérieures au cahier des charges (« CAHIER DE CHARGEEFC &amp; PEP 2021.pdf »), 3,5 % selon le chef comptable (19/10/2026). PEP : 3,5 % (« MANUEL DE PRODUIT D'EPARGNE FPPN VF VF.docx »). Décision fixant le taux appliqué chaque année non reçue.
+Lots 2 et 3 lus le 22/10/2026 : Le rapport de gestion 2025 ne mentionne aucun taux servi ; aucune écriture d'intérêts sur les comptes d'épargne dans le grand livre 2024.</t>
         </is>
       </c>
       <c r="M36" s="76" t="inlineStr">
@@ -1948,7 +1955,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="117" customHeight="1" s="48">
+    <row r="43" ht="162" customHeight="1" s="48">
       <c r="B43" s="70">
         <f>+B42+1</f>
         <v/>
@@ -1977,7 +1984,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Dossiers des programmes immobiliers en attente (liste des immeubles : M. Koffi).
-Nouveaux fichiers du 22/10/2026 : Titres et baux reçus ; valeurs et dernières évaluations non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : certificats de propriété, acte de vente, « CONTRAT DE BAIL SONAPIE N° 2124-03002 / 03037 FPPN.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Titres et baux reçus ; valeurs et dernières évaluations non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : certificats de propriété, acte de vente, « CONTRAT DE BAIL SONAPIE N° 2124-03002 / 03037 FPPN.pdf ».
+Lots 2 et 3 lus le 22/10/2026 : Titres de propriété du siège (Marcory) et du terrain du Plateau reçus ; inventaire et évaluation des biens non reçus.</t>
         </is>
       </c>
       <c r="M43" s="76" t="inlineStr">
@@ -2064,7 +2072,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="147" customHeight="1" s="48">
+    <row r="48" ht="192" customHeight="1" s="48">
       <c r="B48" s="70">
         <f>+B47+1</f>
         <v/>
@@ -2093,7 +2101,8 @@
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
 Pointage des autres équipes (22/10/2026) : Organigramme 2022 (identité et postes) reçu partiellement par l'équipe comptable ; version numérique en attente.
-Nouveaux fichiers du 22/10/2026 : Organigrammes 2020 et 2021 et un courrier de nomination reçus ; contacts des responsables non reçus. Contenu à analyser. Fichiers : « ORGANIGRAMME FPPN 2021(1).pdf » ; 03-Nouveaux Juridiques : « OrganigrammeFPPN_ORI (A) 2020.docx » ; « COURRIER DE NOMINATION DÉFINITIVE.pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : Organigrammes 2020 et 2021 et un courrier de nomination reçus ; contacts des responsables non reçus. Contenu à analyser. Fichiers : « ORGANIGRAMME FPPN 2021(1).pdf » ; 03-Nouveaux Juridiques : « OrganigrammeFPPN_ORI (A) 2020.docx » ; « COURRIER DE NOMINATION DÉFINITIVE.pdf ».
+Lots 2 et 3 lus le 22/10/2026 : Lus : « OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf » ; contacts des responsables non reçus.</t>
         </is>
       </c>
       <c r="M48" s="76" t="inlineStr">
@@ -2422,7 +2431,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="87" customHeight="1" s="48">
+    <row r="59" ht="132" customHeight="1" s="48">
       <c r="B59" s="70">
         <f>+B58+1</f>
         <v/>
@@ -2448,7 +2457,8 @@
       <c r="K59" s="75" t="inlineStr">
         <is>
           <t>Non reçu dans l'envoi du 15/10/2026.
-Pointage des autres équipes (22/10/2026) : Rapports de contrôle de l'AIRMS reçus en version papier par l'équipe comptable ; plan de redressement à rechercher. Copie à obtenir auprès de l'équipe d'audit comptable.</t>
+Pointage des autres équipes (22/10/2026) : Rapports de contrôle de l'AIRMS reçus en version papier par l'équipe comptable ; plan de redressement à rechercher. Copie à obtenir auprès de l'équipe d'audit comptable.
+Lots 2 et 3 lus le 22/10/2026 : Lus : « PLAN D'ACTION 2024.pdf » et « Plan d'action 2025.pdf » ; rapport de contrôle de l'AIRMS et plan de redressement non reçus.</t>
         </is>
       </c>
       <c r="M59" s="76" t="inlineStr">
@@ -2882,7 +2892,7 @@
         </is>
       </c>
     </row>
-    <row r="75" ht="177" customHeight="1" s="48">
+    <row r="75" ht="297" customHeight="1" s="48">
       <c r="B75" s="70">
         <f>+B74+1</f>
         <v/>
@@ -2911,7 +2921,8 @@
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
 Pointage des autres équipes (22/10/2026) : États financiers reçus par l'équipe comptable. Rapports du commissaire aux comptes 2022 à 2025 en attente, 2020 et 2021 à retrouver par le FPPN.
-Nouveaux fichiers du 22/10/2026 : États financiers 2020 au 31/08/2026 reçus ; rapports du commissaire aux comptes et états par risque long non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf », « ETATS FINANCIERS AU 31-08-2026.pdf » (scans) ; « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf ».</t>
+Nouveaux fichiers du 22/10/2026 : États financiers 2020 au 31/08/2026 reçus ; rapports du commissaire aux comptes et états par risque long non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf », « ETATS FINANCIERS AU 31-08-2026.pdf » (scans) ; « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf ».
+Lots 2 et 3 lus le 22/10/2026 : Lus : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf » et « ETATS FINANCIERS AU 31-08-2026.pdf » (scans). Totaux de l'actif brut, résultat et trésorerie identiques aux balances, sauf 2023 (version antérieure : actif brut inférieur de 10 000 000 FCFA, excédent de 928 699 102 contre 930 629 102 FCFA) et résultat au 31/08/2026 (-437 148 460 contre -441 256 500 FCFA). Rapports du commissaire aux comptes et états par risque long non reçus.</t>
         </is>
       </c>
       <c r="M75" s="76" t="inlineStr">
@@ -2989,7 +3000,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="147" customHeight="1" s="48">
+    <row r="78" ht="207" customHeight="1" s="48">
       <c r="B78" s="70">
         <f>+B77+1</f>
         <v/>
@@ -3018,7 +3029,8 @@
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
 Pointage des autres équipes (22/10/2026) : PV d'AG reçus par l'équipe comptable sauf 2020 et 2023 : l'affectation de 2023 reste à obtenir. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : AG du 15/02/2024 : affectation à vérifier ; origine du compte 10620000 non documentée. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan).</t>
+Nouveaux fichiers du 22/10/2026 : AG du 15/02/2024 : affectation à vérifier ; origine du compte 10620000 non documentée. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan).
+Lots 2 et 3 lus le 22/10/2026 : Le rapport de gestion 2023 corrigé propose l'affectation de l'excédent 2023 (36 % aux réserves obligatoires, 20 % aux réserves libres, 44 % au déficit cumulé) ; PV d'AG non reçus.</t>
         </is>
       </c>
       <c r="M78" s="76" t="inlineStr">
@@ -3095,7 +3107,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="162" customHeight="1" s="48">
+    <row r="81" ht="222" customHeight="1" s="48">
       <c r="B81" s="70">
         <f>+B80+1</f>
         <v/>
@@ -3124,7 +3136,8 @@
         <is>
           <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
 Pointage des autres équipes (22/10/2026) : Procès-verbaux des AG, CA et commissions reçus par l'équipe comptable, sauf 2020 et 2023. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : PV de 2024 et compositions des organes reçus ; calendrier statutaire et autres PV à compléter. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » ; listes des administrateurs et membres de la commission de surveillance.</t>
+Nouveaux fichiers du 22/10/2026 : PV de 2024 et compositions des organes reçus ; calendrier statutaire et autres PV à compléter. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » ; listes des administrateurs et membres de la commission de surveillance.
+Lots 2 et 3 lus le 22/10/2026 : Lus : listes des administrateurs et des membres de la commission de surveillance et de contrôle d'août 2020 et d'août 2023 (scans) ; calendrier et PV des réunions non reçus.</t>
         </is>
       </c>
       <c r="M81" s="76" t="inlineStr">
@@ -3167,7 +3180,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="42" customHeight="1" s="48">
+    <row r="83" ht="87" customHeight="1" s="48">
       <c r="B83" s="70">
         <f>+B82+1</f>
         <v/>
@@ -3188,16 +3201,19 @@
       <c r="H83" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I83" s="73" t="n"/>
+      <c r="I83" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J83" s="74" t="n"/>
       <c r="K83" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).</t>
+          <t>Demande issue de la lecture des textes de l'AIRMS (rapport v3, partie 10).
+Lots 2 et 3 lus le 22/10/2026 : Le rapport de gestion 2023 corrigé nomme la structure : Centre Médical du Policier (CMP). Statut juridique non reçu.</t>
         </is>
       </c>
       <c r="M83" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4101,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="42" customHeight="1" s="48">
+    <row r="111" ht="102" customHeight="1" s="48">
       <c r="B111" s="70">
         <f>+B110+1</f>
         <v/>
@@ -4106,16 +4122,19 @@
       <c r="H111" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I111" s="73" t="n"/>
+      <c r="I111" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J111" s="74" t="n"/>
       <c r="K111" s="75" t="inlineStr">
         <is>
-          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.</t>
+          <t>Revue des provisions (rapport v5) : analyse en attente de ce document.
+Lots 2 et 3 lus le 22/10/2026 : La convention IPS-CGRAE confirme la garantie santé des retraités souscripteurs ; durée, cotisation et ayants droit couverts non précisés (« CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf »).</t>
         </is>
       </c>
       <c r="M111" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4286,7 +4305,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="162" customHeight="1" s="48">
+    <row r="118" ht="237" customHeight="1" s="48">
       <c r="B118" s="70">
         <f>+B117+1</f>
         <v/>
@@ -4315,7 +4334,8 @@
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : Titres de propriété et tableau de synthèse des biens en attente (M. Sangaré).
-Nouveaux fichiers du 22/10/2026 : Deux certificats de propriété et un acte de vente reçus ; situation de chaque terrain (projet, attribution, litige) non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « Certificat de Propriété Terrain Marcori (Siège).pdf » ; « Certificat de Propriété Terrain Plateau.pdf » ; « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE… ».</t>
+Nouveaux fichiers du 22/10/2026 : Deux certificats de propriété et un acte de vente reçus ; situation de chaque terrain (projet, attribution, litige) non reçue. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « Certificat de Propriété Terrain Marcori (Siège).pdf » ; « Certificat de Propriété Terrain Plateau.pdf » ; « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE… ».
+Lots 2 et 3 lus le 22/10/2026 : Lus : « Certificat de Propriété Terrain Marcori (Siège).pdf », « Certificat de Propriété Terrain Plateau.pdf » et « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE AU PROFIT DU FPPN.pdf » (lot n° 40 de 1 469 m²). Scans partiellement lisibles ; situation et valeur de chaque terrain non reçues.</t>
         </is>
       </c>
       <c r="M118" s="76" t="inlineStr">
@@ -4324,7 +4344,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="42" customHeight="1" s="48">
+    <row r="119" ht="102" customHeight="1" s="48">
       <c r="B119" s="70">
         <f>+B118+1</f>
         <v/>
@@ -4345,16 +4365,19 @@
       <c r="H119" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I119" s="73" t="n"/>
+      <c r="I119" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J119" s="74" t="n"/>
       <c r="K119" s="75" t="inlineStr">
         <is>
-          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).</t>
+          <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
+Lots 2 et 3 lus le 22/10/2026 : Lus : « CONTRAT DE BAIL SONAPIE N° 2124-03002 FPPN.pdf » et « … 2124-03037 FPPN.pdf » (scans peu lisibles, bail de deux ans, loyer trimestriel) ; objet à rapprocher des immeubles d'Aboisso, encaissements non reçus.</t>
         </is>
       </c>
       <c r="M119" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
+          <t>Partiellement Reçu</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4449,7 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="102" customHeight="1" s="48">
+    <row r="122" ht="147" customHeight="1" s="48">
       <c r="B122" s="70">
         <f>+B121+1</f>
         <v/>
@@ -4458,7 +4481,8 @@
       <c r="K122" s="75" t="inlineStr">
         <is>
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
-Nouveaux fichiers du 22/10/2026 : Convention de la clinique (CMP) avec Transvie reçue ; bilan d'ouverture et détail des comptes 47111104 et 47111105 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf » (scan).</t>
+Nouveaux fichiers du 22/10/2026 : Convention de la clinique (CMP) avec Transvie reçue ; bilan d'ouverture et détail des comptes 47111104 et 47111105 non reçus. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « CONVENTION TRANSVIE-CMP.pdf » (scan).
+Lots 2 et 3 lus le 22/10/2026 : Lu : « CONVENTION TRANSVIE-CMP.pdf » (soins du CMP aux assurés de Transvie sur lettre de garantie) ; bilan d'ouverture du CMP non reçu.</t>
         </is>
       </c>
       <c r="M122" s="76" t="inlineStr">
@@ -4775,7 +4799,7 @@
         </is>
       </c>
     </row>
-    <row r="133" ht="207" customHeight="1" s="48">
+    <row r="133" ht="252" customHeight="1" s="48">
       <c r="B133" s="70">
         <f>+B132+1</f>
         <v/>
@@ -4809,7 +4833,8 @@
           <t>Demande issue des entretiens du 19/10/2026 avec le chef comptable (PBC complémentaire placements et provisions).
 Pointage des autres équipes (22/10/2026) : DISA et état 301 reçus sauf 2026 ; ITS et FDFP reçus (2021 manquant) ; déclarations CNPS en attente. Copie à obtenir auprès de l'équipe d'audit comptable.
 Nouveaux fichiers du 22/10/2026 : DISA, état 301 et appels CNPS annuels reçus pour 2020 à 2025 ; déclarations mensuelles CNPS et 2026 non reçues. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : « ETAT 301 &amp; DISA 2020 à 2025 FPPN.xls », « DISA_256927_2021 à 2025.xls », DASC 2022, 2023, 2025.
-Lot 1 lu le 22/10/2026 : Lu : états 301 et DISA 2020 à 2025, appels CNPS annuels, DASC 2022, 2023, 2025, fichiers e-CNPS complémentaires 2022. Déclarations mensuelles CNPS et 2026 non reçues.</t>
+Lot 1 lu le 22/10/2026 : Lu : états 301 et DISA 2020 à 2025, appels CNPS annuels, DASC 2022, 2023, 2025, fichiers e-CNPS complémentaires 2022. Déclarations mensuelles CNPS et 2026 non reçues.
+Lots 2 et 3 lus le 22/10/2026 : Lot 3 : DISA et DASC 2021 à 2025 scannées et états des travailleurs occasionnels 2024 et 2025, en double des fichiers Excel du lot 1.</t>
         </is>
       </c>
       <c r="M133" s="76" t="inlineStr">
@@ -5039,7 +5064,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="237" customHeight="1" s="48">
+    <row r="143" ht="297" customHeight="1" s="48">
       <c r="B143" s="70">
         <f>+B140+1</f>
         <v/>
@@ -5073,7 +5098,8 @@
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : Mouvements du personnel et livres de paie en attente (M. Koffi) : le statut civil ou policier devra y figurer.
 Nouveaux fichiers du 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS (personnel civil) ; les fonctionnaires de police en service n'y figurent a priori pas. Statut à confirmer. Contenu à analyser. Fichiers : 04-Nouveaux Personnel et paie : DISA 2021 à 2025 ; « RECAPSALAIRES » des états 301.
-Lot 1 lu le 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS. Les états 301 distinguent des onglets « RECAPSALAIRES 2024 CMP » et « RECAPSALAIRES 2025 GRENIER » : Direction Générale, clinique et Grenier sont identifiables par nom. Le statut des policiers en service n'y figure pas.</t>
+Lot 1 lu le 22/10/2026 : Les DISA couvrent les salariés déclarés à la CNPS. Les états 301 distinguent des onglets « RECAPSALAIRES 2024 CMP » et « RECAPSALAIRES 2025 GRENIER » : Direction Générale, clinique et Grenier sont identifiables par nom. Le statut des policiers en service n'y figure pas.
+Lots 2 et 3 lus le 22/10/2026 : Organigrammes reçus ; le statut civil ou policier de chaque agent n'y figure pas. Rattachement aux entités établi par les récapitulatifs de salaires 2024 (CMP) et 2025 (Grenier).</t>
         </is>
       </c>
       <c r="M143" s="76" t="inlineStr">
@@ -5194,7 +5220,7 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="147" customHeight="1" s="48">
+    <row r="149" ht="192" customHeight="1" s="48">
       <c r="B149" s="70">
         <f>+B148+1</f>
         <v/>
@@ -5223,7 +5249,8 @@
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
 Pointage des autres équipes (22/10/2026) : PV d'AG reçus par l'équipe comptable, sauf 2020 et 2023 ; affectations des résultats à y vérifier. Copie à obtenir auprès de l'équipe d'audit comptable.
-Nouveaux fichiers du 22/10/2026 : PV de l'AG ordinaire du 15/02/2024 reçu ; autres AG d'affectation non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan).</t>
+Nouveaux fichiers du 22/10/2026 : PV de l'AG ordinaire du 15/02/2024 reçu ; autres AG d'affectation non reçues. Contenu à analyser. Fichiers : 03-Nouveaux Juridiques : « PV AG ORDINAIRE DU 15 FEVRIER 2024.pdf » (scan).
+Lots 2 et 3 lus le 22/10/2026 : Propositions d'affectation lues dans les rapports de gestion ; PV d'AG d'approbation de 2020 à 2025 non reçus.</t>
         </is>
       </c>
       <c r="M149" s="76" t="inlineStr">
@@ -5232,7 +5259,7 @@
         </is>
       </c>
     </row>
-    <row r="150" ht="57" customHeight="1" s="48">
+    <row r="150" ht="87" customHeight="1" s="48">
       <c r="B150" s="70">
         <f>+B149+1</f>
         <v/>
@@ -5253,20 +5280,23 @@
       <c r="H150" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I150" s="73" t="n"/>
+      <c r="I150" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J150" s="74" t="n"/>
       <c r="K150" s="75" t="inlineStr">
         <is>
-          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).</t>
+          <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
+Lots 2 et 3 lus le 22/10/2026 : La convention IPS-CGRAE organise la couverture santé des policiers retraités ; la décision des organes sur la qualité de membre des retraités reste à recevoir.</t>
         </is>
       </c>
       <c r="M150" s="76" t="inlineStr">
         <is>
-          <t>Non Reçu</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="72" customHeight="1" s="48">
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="132" customHeight="1" s="48">
       <c r="B151" s="70">
         <f>+B150+1</f>
         <v/>
@@ -5287,15 +5317,195 @@
       <c r="H151" s="73" t="n">
         <v>46321</v>
       </c>
-      <c r="I151" s="73" t="n"/>
+      <c r="I151" s="73" t="n">
+        <v>46317</v>
+      </c>
       <c r="J151" s="74" t="n"/>
       <c r="K151" s="75" t="inlineStr">
         <is>
           <t>Demande issue de la lecture des statuts et du règlement intérieur du 15/06/2023 (PBC complémentaire textes et personnel).
-Pointage des autres équipes (22/10/2026) : À rechercher dans les PV du CA reçus par l'équipe comptable.</t>
+Pointage des autres équipes (22/10/2026) : À rechercher dans les PV du CA reçus par l'équipe comptable.
+Lots 2 et 3 lus le 22/10/2026 : Organigrammes 2020 et 2021 reçus (« OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf ») ; délibération approuvant le cadre organique non reçue.</t>
         </is>
       </c>
       <c r="M151" s="76" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="18" customHeight="1" s="48">
+      <c r="C152" s="69" t="inlineStr">
+        <is>
+          <t>Documents reçus le 22/10/2026 (demandes issues du rapport v9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="87" customHeight="1" s="48">
+      <c r="B153" s="70">
+        <f>+B151+1</f>
+        <v/>
+      </c>
+      <c r="C153" s="71" t="inlineStr">
+        <is>
+          <t>Version des comptes 2023 approuvée par l'Assemblée générale (les états financiers scannés portent un actif brut de 16 157 155 123 FCFA et un excédent de 928 699 102 FCFA, la balance et le rapport de gestion corrigé 16 167 155 123 FCFA et 930 629 102 FCFA) et explication de l'écart de résultat au 31/08/2026 (états financiers -437 148 460 FCFA, balance -441 256 500 FCFA).</t>
+        </is>
+      </c>
+      <c r="E153" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G153" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H153" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I153" s="73" t="n"/>
+      <c r="J153" s="74" t="n"/>
+      <c r="K153" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+        </is>
+      </c>
+      <c r="M153" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="75" customHeight="1" s="48">
+      <c r="B154" s="70">
+        <f>+B153+1</f>
+        <v/>
+      </c>
+      <c r="C154" s="71" t="inlineStr">
+        <is>
+          <t>Clé de répartition maladie (936) / décès (8Z6) appliquée en janvier et février 2024 (rapport médian 8Z6 / 936 de 0,3059 et 0,3023, contre 0,3263 ensuite) et liste des dix adhérents d'écart entre l'étude des ratios et les fichiers 8Z6 de janvier à juin 2026.</t>
+        </is>
+      </c>
+      <c r="E154" s="72" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="G154" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H154" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I154" s="73" t="n"/>
+      <c r="J154" s="74" t="n"/>
+      <c r="K154" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+        </is>
+      </c>
+      <c r="M154" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="75" customHeight="1" s="48">
+      <c r="B155" s="70">
+        <f>+B154+1</f>
+        <v/>
+      </c>
+      <c r="C155" s="71" t="inlineStr">
+        <is>
+          <t>Rapport de gestion 2025 rectifié présentant le solde de l'épargne due aux mutualistes au 31/12/2025 (PEP et EFC), distinct des cotisations collectées dans l'année (4 387 823 635 FCFA présentés comme l'épargne au 31/12/2025).</t>
+        </is>
+      </c>
+      <c r="E155" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G155" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H155" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I155" s="73" t="n"/>
+      <c r="J155" s="74" t="n"/>
+      <c r="K155" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue du rapport v9 (partie 6).</t>
+        </is>
+      </c>
+      <c r="M155" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="75" customHeight="1" s="48">
+      <c r="B156" s="70">
+        <f>+B155+1</f>
+        <v/>
+      </c>
+      <c r="C156" s="71" t="inlineStr">
+        <is>
+          <t>Personnel : âge de départ à la retraite appliqué, nombre d'enfants à charge de chaque salarié, justification des douze dates d'embauche modifiées dans la DISA 2025, rattachement (DG, CMP, Grenier) des dix-neuf agents recrutés en 2025, note de calcul du compte 196 (complète les items 78 et 98).</t>
+        </is>
+      </c>
+      <c r="E156" s="72" t="inlineStr">
+        <is>
+          <t>Urgent</t>
+        </is>
+      </c>
+      <c r="G156" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H156" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I156" s="73" t="n"/>
+      <c r="J156" s="74" t="n"/>
+      <c r="K156" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue du recalcul de la provision du personnel (rapport v9, partie 9).</t>
+        </is>
+      </c>
+      <c r="M156" s="76" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="75" customHeight="1" s="48">
+      <c r="B157" s="70">
+        <f>+B156+1</f>
+        <v/>
+      </c>
+      <c r="C157" s="71" t="inlineStr">
+        <is>
+          <t>Annexe 2 de la convention IPS-CGRAE (bulletin de souscription), barème de la cotisation des retraités et liste des retraités souscripteurs non précomptés faute de quotité cessible suffisante.</t>
+        </is>
+      </c>
+      <c r="E157" s="72" t="inlineStr">
+        <is>
+          <t>Moyen</t>
+        </is>
+      </c>
+      <c r="G157" s="73" t="n">
+        <v>46317</v>
+      </c>
+      <c r="H157" s="73" t="n">
+        <v>46324</v>
+      </c>
+      <c r="I157" s="73" t="n"/>
+      <c r="J157" s="74" t="n"/>
+      <c r="K157" s="75" t="inlineStr">
+        <is>
+          <t>Demande issue de la lecture de la convention IPS-CGRAE (rapport v9, partie 8).</t>
+        </is>
+      </c>
+      <c r="M157" s="76" t="inlineStr">
         <is>
           <t>Non Reçu</t>
         </is>
@@ -5308,7 +5518,7 @@
     <mergeCell ref="C5:M5"/>
     <mergeCell ref="C4:M4"/>
   </mergeCells>
-  <conditionalFormatting sqref="M11:M151">
+  <conditionalFormatting sqref="M11:M157">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="6" text="" percent="0" bottom="0">
       <formula>"Partiellement Reçu"</formula>
     </cfRule>
@@ -5319,7 +5529,7 @@
       <formula>"Reçu"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E11:E151">
+  <conditionalFormatting sqref="E11:E157">
     <cfRule type="cellIs" rank="0" priority="5" equalAverage="0" operator="equal" aboveAverage="0" dxfId="9" text="" percent="0" bottom="0">
       <formula>"Faible"</formula>
     </cfRule>
@@ -5358,6 +5568,722 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B2:F31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" style="48" min="2" max="2"/>
+    <col width="48" customWidth="1" style="48" min="3" max="3"/>
+    <col width="16" customWidth="1" style="48" min="4" max="4"/>
+    <col width="16" customWidth="1" style="48" min="5" max="5"/>
+    <col width="100" customWidth="1" style="48" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="97" t="inlineStr">
+        <is>
+          <t>Pointage sur le contenu des lots 2 et 3 des nouveaux fichiers (22/10/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1" s="48">
+      <c r="B3" s="79" t="inlineStr">
+        <is>
+          <t>Lot 2 : 26 fichiers, lot 3 : 29 fichiers, empreintes SHA-256 conformes aux journaux « journal_lot2.csv » et « journal_lot3.csv ». Les scans ont été lus par reconnaissance de caractères et les montants cités vérifiés sur l'image. Reçus sans item de la PBC : budgets de 2020 à 2026, PV d'arrêté de caisse de 2020 au 26/08/2026, convention DEPA. Items 110 à 114 ajoutés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="80" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C5" s="80" t="inlineStr">
+        <is>
+          <t>Document demandé (PBC actuarielle)</t>
+        </is>
+      </c>
+      <c r="D5" s="80" t="inlineStr">
+        <is>
+          <t>Statut avant</t>
+        </is>
+      </c>
+      <c r="E5" s="80" t="inlineStr">
+        <is>
+          <t>Statut après</t>
+        </is>
+      </c>
+      <c r="F5" s="80" t="inlineStr">
+        <is>
+          <t>Constat sur le contenu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1" s="48">
+      <c r="B6" s="96" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="95" t="inlineStr">
+        <is>
+          <t>Convention conclue avec la CGRAE pour la prise en charge des retraités, et ses avenants.</t>
+        </is>
+      </c>
+      <c r="D6" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E6" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F6" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf » (scan) : précompte sur pension des cotisations de prise en charge médicale (art. 3), pas de suspension des soins pour retard de la CGRAE (art. 4.1 e), précompte dans la limite de la quotité cessible (art. 4.2 a), aucun frais de gestion (art. 5). Annexe 2 (bulletin de souscription) et montant de la cotisation non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1" s="48">
+      <c r="B7" s="96" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" s="95" t="inlineStr">
+        <is>
+          <t>Détail des provisions inscrites au bilan, par nature et par garantie, au 31/12/2019, 31/12/2020, 31/12/2021, 31/12/2022, 31/12/2023, 31/12/2024, 31/12/2025 et 3</t>
+        </is>
+      </c>
+      <c r="D7" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E7" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F7" s="95" t="inlineStr">
+        <is>
+          <t>Les états financiers 2020 au 31/08/2026 montrent les provisions au passif sans détail par garantie (« ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf » et « ETATS FINANCIERS AU 31-08-2026.pdf »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1" s="48">
+      <c r="B8" s="96" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>Tout rapport actuariel, étude technique ou note de calcul des engagements envers les mutualistes existant, quelle que soit sa date.</t>
+        </is>
+      </c>
+      <c r="D8" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E8" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>Lus : rapports de gestion et rapports moraux 2020 à 2025 (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf ») : analyses de l'excédent et de l'épargne, sans calcul actuariel des engagements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1" s="48">
+      <c r="B9" s="96" t="n">
+        <v>12</v>
+      </c>
+      <c r="C9" s="95" t="inlineStr">
+        <is>
+          <t>Cotisations appelées et cotisations encaissées par mois et par catégorie de membres, du 01/01/2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="D9" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E9" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F9" s="95" t="inlineStr">
+        <is>
+          <t>Les rapports de gestion donnent les cotisations maladie annuelles (« Cotisation Maladie (3,5 % SB) »), sans détail mensuel ni par catégorie (« RAPPORT DE GESTION 2020 FPPN - BASE - 10 (A).docx », « 1- RAPPORT MORAL 30 juin 2021 définitif (A).docx », « RAPPORT MORAL 2022 (définitif) (A).docx », « BILAN_DE_L'EXERCICE_CLOS_31.12.2023_(corrigé_et_finalisé)[1].pdf », « RAPPORT DE GESTION DETAILLE EXERCICE 2024.pdf », « RAPPORT GESTION NOUVEAUpdf.pdf », « Rapport de Gestion  2025 Final (2).pdf »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1" s="48">
+      <c r="B10" s="96" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" s="95" t="inlineStr">
+        <is>
+          <t>Taux d'intérêt crédité sur l'épargne chaque année et décision qui l'a fixé.</t>
+        </is>
+      </c>
+      <c r="D10" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E10" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F10" s="95" t="inlineStr">
+        <is>
+          <t>Le rapport de gestion 2025 ne mentionne aucun taux servi ; aucune écriture d'intérêts sur les comptes d'épargne dans le grand livre 2024.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1" s="48">
+      <c r="B11" s="96" t="n">
+        <v>23</v>
+      </c>
+      <c r="C11" s="95" t="inlineStr">
+        <is>
+          <t>Biens immobiliers et participations (centre médical, programme immobilier, autres) au 31/08/2026 : valeur au bilan, dernière évaluation, revenus annuels, contra</t>
+        </is>
+      </c>
+      <c r="D11" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E11" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F11" s="95" t="inlineStr">
+        <is>
+          <t>Titres de propriété du siège (Marcory) et du terrain du Plateau reçus ; inventaire et évaluation des biens non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1" s="48">
+      <c r="B12" s="96" t="n">
+        <v>26</v>
+      </c>
+      <c r="C12" s="95" t="inlineStr">
+        <is>
+          <t>Nom, fonction et contact des responsables à rencontrer pour les prestations, l'épargne, les placements et les données des mutualistes.</t>
+        </is>
+      </c>
+      <c r="D12" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E12" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F12" s="95" t="inlineStr">
+        <is>
+          <t>Lus : « OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf » ; contacts des responsables non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1" s="48">
+      <c r="B13" s="96" t="n">
+        <v>35</v>
+      </c>
+      <c r="C13" s="95" t="inlineStr">
+        <is>
+          <t>Rapport de contrôle de l'AIRMS et plan de redressement en cours.</t>
+        </is>
+      </c>
+      <c r="D13" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E13" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F13" s="95" t="inlineStr">
+        <is>
+          <t>Lus : « PLAN D'ACTION 2024.pdf » et « Plan d'action 2025.pdf » ; rapport de contrôle de l'AIRMS et plan de redressement non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1" s="48">
+      <c r="B14" s="96" t="n">
+        <v>47</v>
+      </c>
+      <c r="C14" s="95" t="inlineStr">
+        <is>
+          <t>Rapports du commissaire aux comptes 2020 à 2025 et états financiers par risque long (règlement d'exécution n° 004/2022, art. 12 et 13).</t>
+        </is>
+      </c>
+      <c r="D14" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E14" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F14" s="95" t="inlineStr">
+        <is>
+          <t>Lus : « ETATS FINANCIERS 2020.pdf » à « ETATS FINANCIERS 2025.pdf » et « ETATS FINANCIERS AU 31-08-2026.pdf » (scans). Totaux de l'actif brut, résultat et trésorerie identiques aux balances, sauf 2023 (version antérieure : actif brut inférieur de 10 000 000 FCFA, excédent de 928 699 102 contre 930 629 102 FCFA) et résultat au 31/08/2026 (-437 148 460 contre -441 256 500 FCFA). Rapports du commissaire aux comptes et états par risque long non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1" s="48">
+      <c r="B15" s="96" t="n">
+        <v>50</v>
+      </c>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>PV d'AG d'affectation des excédents 2023 à 2025 et origine du compte 10620000 « Réserve disponible ».</t>
+        </is>
+      </c>
+      <c r="D15" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E15" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F15" s="95" t="inlineStr">
+        <is>
+          <t>Le rapport de gestion 2023 corrigé propose l'affectation de l'excédent 2023 (36 % aux réserves obligatoires, 20 % aux réserves libres, 44 % au déficit cumulé) ; PV d'AG non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1" s="48">
+      <c r="B16" s="96" t="n">
+        <v>53</v>
+      </c>
+      <c r="C16" s="95" t="inlineStr">
+        <is>
+          <t>Calendrier statutaire et PV des réunions du conseil, de l'organe de contrôle et de l'AG, 2022 à 2025.</t>
+        </is>
+      </c>
+      <c r="D16" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E16" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F16" s="95" t="inlineStr">
+        <is>
+          <t>Lus : listes des administrateurs et des membres de la commission de surveillance et de contrôle d'août 2020 et d'août 2023 (scans) ; calendrier et PV des réunions non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1" s="48">
+      <c r="B17" s="96" t="n">
+        <v>55</v>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
+        <is>
+          <t>Dénomination complète et statut juridique de la structure désignée « CMP » dans les comptes 47111104 et 47111105, et comptabilité séparée de ses activités.</t>
+        </is>
+      </c>
+      <c r="D17" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E17" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F17" s="95" t="inlineStr">
+        <is>
+          <t>Le rapport de gestion 2023 corrigé nomme la structure : Centre Médical du Policier (CMP). Statut juridique non reçu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1" s="48">
+      <c r="B18" s="96" t="n">
+        <v>79</v>
+      </c>
+      <c r="C18" s="95" t="inlineStr">
+        <is>
+          <t>Règles de la garantie santé des retraités : durée (à vie ou limitée), conditions, cotisation, décision qui la fonde.</t>
+        </is>
+      </c>
+      <c r="D18" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E18" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F18" s="95" t="inlineStr">
+        <is>
+          <t>La convention IPS-CGRAE confirme la garantie santé des retraités souscripteurs ; durée, cotisation et ayants droit couverts non précisés (« CONVENTION DE PARTENARIAT ENTRE IPS-CGRAE ET LE FPPN.pdf »).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1" s="48">
+      <c r="B19" s="96" t="n">
+        <v>84</v>
+      </c>
+      <c r="C19" s="95" t="inlineStr">
+        <is>
+          <t>Titres de propriété ou actes d'acquisition des terrains, situation de chaque terrain (projet, attribution, litige).</t>
+        </is>
+      </c>
+      <c r="D19" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E19" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F19" s="95" t="inlineStr">
+        <is>
+          <t>Lus : « Certificat de Propriété Terrain Marcori (Siège).pdf », « Certificat de Propriété Terrain Plateau.pdf » et « Vente ferme par les consorts SIRANSY TOURE SOULEYMANE AU PROFIT DU FPPN.pdf » (lot n° 40 de 1 469 m²). Scans partiellement lisibles ; situation et valeur de chaque terrain non reçues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1" s="48">
+      <c r="B20" s="96" t="n">
+        <v>85</v>
+      </c>
+      <c r="C20" s="95" t="inlineStr">
+        <is>
+          <t>Baux et encaissements des immeubles d'Aboisso.</t>
+        </is>
+      </c>
+      <c r="D20" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E20" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F20" s="95" t="inlineStr">
+        <is>
+          <t>Lus : « CONTRAT DE BAIL SONAPIE N° 2124-03002 FPPN.pdf » et « … 2124-03037 FPPN.pdf » (scans peu lisibles, bail de deux ans, loyer trimestriel) ; objet à rapprocher des immeubles d'Aboisso, encaissements non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1" s="48">
+      <c r="B21" s="96" t="n">
+        <v>88</v>
+      </c>
+      <c r="C21" s="95" t="inlineStr">
+        <is>
+          <t>Bilan d'ouverture de la clinique du FPPN (CMP) et détail des comptes 47111104 et 47111105.</t>
+        </is>
+      </c>
+      <c r="D21" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E21" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F21" s="95" t="inlineStr">
+        <is>
+          <t>Lu : « CONVENTION TRANSVIE-CMP.pdf » (soins du CMP aux assurés de Transvie sur lettre de garantie) ; bilan d'ouverture du CMP non reçu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1" s="48">
+      <c r="B22" s="96" t="n">
+        <v>97</v>
+      </c>
+      <c r="C22" s="95" t="inlineStr">
+        <is>
+          <t>Déclarations CNPS de 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="D22" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E22" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F22" s="95" t="inlineStr">
+        <is>
+          <t>Lot 3 : DISA et DASC 2021 à 2025 scannées et états des travailleurs occasionnels 2024 et 2025, en double des fichiers Excel du lot 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1" s="48">
+      <c r="B23" s="96" t="n">
+        <v>103</v>
+      </c>
+      <c r="C23" s="95" t="inlineStr">
+        <is>
+          <t>Fichier du personnel de la Direction Générale avec une colonne de statut : personnel civil salarié ou fonctionnaire de police en service (article 31 du règlemen</t>
+        </is>
+      </c>
+      <c r="D23" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E23" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F23" s="95" t="inlineStr">
+        <is>
+          <t>Organigrammes reçus ; le statut civil ou policier de chaque agent n'y figure pas. Rattachement aux entités établi par les récapitulatifs de salaires 2024 (CMP) et 2025 (Grenier).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1" s="48">
+      <c r="B24" s="96" t="n">
+        <v>107</v>
+      </c>
+      <c r="C24" s="95" t="inlineStr">
+        <is>
+          <t>Procès-verbaux des Assemblées Générales d'affectation des résultats de 2020 à 2025 (article 90 des statuts : réserve légale de 20 % à 50 % de l'excédent net).</t>
+        </is>
+      </c>
+      <c r="D24" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="E24" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F24" s="95" t="inlineStr">
+        <is>
+          <t>Propositions d'affectation lues dans les rapports de gestion ; PV d'AG d'approbation de 2020 à 2025 non reçus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1" s="48">
+      <c r="B25" s="96" t="n">
+        <v>108</v>
+      </c>
+      <c r="C25" s="95" t="inlineStr">
+        <is>
+          <t>Décision fixant la situation des policiers retraités : maintien de la qualité de membre (article 7 des statuts), restitution de la carte (article 38 du règlemen</t>
+        </is>
+      </c>
+      <c r="D25" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E25" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F25" s="95" t="inlineStr">
+        <is>
+          <t>La convention IPS-CGRAE organise la couverture santé des policiers retraités ; la décision des organes sur la qualité de membre des retraités reste à recevoir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1" s="48">
+      <c r="B26" s="96" t="n">
+        <v>109</v>
+      </c>
+      <c r="C26" s="95" t="inlineStr">
+        <is>
+          <t>Délibération du Conseil d'Administration approuvant le cadre organique des emplois de la Direction Générale et la grille des salaires et indemnités (articles 61</t>
+        </is>
+      </c>
+      <c r="D26" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="E26" s="95" t="inlineStr">
+        <is>
+          <t>Partiellement Reçu</t>
+        </is>
+      </c>
+      <c r="F26" s="95" t="inlineStr">
+        <is>
+          <t>Organigrammes 2020 et 2021 reçus (« OrganigrammeFPPN_ORI (A) 2020.docx », « ORGANIGRAMME FPPN 2021(1).pdf », « COURRIER DE NOMINATION DÉFINITIVE.pdf ») ; délibération approuvant le cadre organique non reçue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1" s="48">
+      <c r="B27" s="96" t="n">
+        <v>110</v>
+      </c>
+      <c r="C27" s="95" t="inlineStr">
+        <is>
+          <t>Version des comptes 2023 approuvée par l'Assemblée générale (les états financiers scannés portent un actif brut de 16 157 155 123 FCFA et un excédent de 928 699</t>
+        </is>
+      </c>
+      <c r="D27" s="95" t="inlineStr">
+        <is>
+          <t>Nouveau</t>
+        </is>
+      </c>
+      <c r="E27" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="F27" s="95" t="inlineStr">
+        <is>
+          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1" s="48">
+      <c r="B28" s="96" t="n">
+        <v>111</v>
+      </c>
+      <c r="C28" s="95" t="inlineStr">
+        <is>
+          <t>Clé de répartition maladie (936) / décès (8Z6) appliquée en janvier et février 2024 (rapport médian 8Z6 / 936 de 0,3059 et 0,3023, contre 0,3263 ensuite) et lis</t>
+        </is>
+      </c>
+      <c r="D28" s="95" t="inlineStr">
+        <is>
+          <t>Nouveau</t>
+        </is>
+      </c>
+      <c r="E28" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="F28" s="95" t="inlineStr">
+        <is>
+          <t>Demande issue des contrôles croisés du rapport v9 (partie 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1" s="48">
+      <c r="B29" s="96" t="n">
+        <v>112</v>
+      </c>
+      <c r="C29" s="95" t="inlineStr">
+        <is>
+          <t>Rapport de gestion 2025 rectifié présentant le solde de l'épargne due aux mutualistes au 31/12/2025 (PEP et EFC), distinct des cotisations collectées dans l'ann</t>
+        </is>
+      </c>
+      <c r="D29" s="95" t="inlineStr">
+        <is>
+          <t>Nouveau</t>
+        </is>
+      </c>
+      <c r="E29" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="F29" s="95" t="inlineStr">
+        <is>
+          <t>Demande issue du rapport v9 (partie 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1" s="48">
+      <c r="B30" s="96" t="n">
+        <v>113</v>
+      </c>
+      <c r="C30" s="95" t="inlineStr">
+        <is>
+          <t>Personnel : âge de départ à la retraite appliqué, nombre d'enfants à charge de chaque salarié, justification des douze dates d'embauche modifiées dans la DISA 2</t>
+        </is>
+      </c>
+      <c r="D30" s="95" t="inlineStr">
+        <is>
+          <t>Nouveau</t>
+        </is>
+      </c>
+      <c r="E30" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="F30" s="95" t="inlineStr">
+        <is>
+          <t>Demande issue du recalcul de la provision du personnel (rapport v9, partie 9).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1" s="48">
+      <c r="B31" s="96" t="n">
+        <v>114</v>
+      </c>
+      <c r="C31" s="95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Annexe 2 de la convention IPS-CGRAE (bulletin de souscription), barème de la cotisation des retraités et liste des retraités souscripteurs non précomptés faute </t>
+        </is>
+      </c>
+      <c r="D31" s="95" t="inlineStr">
+        <is>
+          <t>Nouveau</t>
+        </is>
+      </c>
+      <c r="E31" s="95" t="inlineStr">
+        <is>
+          <t>Non Reçu</t>
+        </is>
+      </c>
+      <c r="F31" s="95" t="inlineStr">
+        <is>
+          <t>Demande issue de la lecture de la convention IPS-CGRAE (rapport v9, partie 8).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B3:F3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -5432,7 +6358,7 @@
       </c>
       <c r="D7" s="95" t="inlineStr">
         <is>
-          <t>1, 3, 4, 6, 7, 8, 9, 12, 13, 17, 18, 20, 21, 23, 26, 27, 28, 30, 34, 35, 37, 42, 44, 47, 50, 53, 57, 71, 73, 76, 80, 83, 84, 88, 91, 97, 99, 103, 107</t>
+          <t>1, 3, 4, 6, 7, 8, 9, 12, 13, 17, 18, 20, 21, 23, 26, 27, 28, 30, 34, 35, 37, 42, 44, 47, 50, 53, 55, 57, 71, 73, 76, 79, 80, 83, 84, 85, 88, 91, 97, 99, 103, 107, 108, 109</t>
         </is>
       </c>
     </row>
@@ -5448,7 +6374,7 @@
       </c>
       <c r="D8" s="95" t="inlineStr">
         <is>
-          <t>5, 10, 11, 14, 15, 19, 22, 24, 25, 29, 31, 32, 36, 38, 39, 40, 41, 43, 48, 49, 51, 52, 54, 55, 56, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 72, 75, 77, 78, 79, 81, 82, 85, 86, 87, 89, 92, 94, 95, 96, 98, 104, 105, 106, 108, 109</t>
+          <t>5, 10, 11, 14, 15, 19, 22, 24, 25, 29, 31, 32, 36, 38, 39, 40, 41, 43, 48, 49, 51, 52, 54, 56, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 72, 75, 77, 78, 81, 82, 86, 87, 89, 92, 94, 95, 96, 98, 104, 105, 106, 110, 111, 112, 113, 114</t>
         </is>
       </c>
     </row>
@@ -42734,7 +43660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E51"/>
+  <dimension ref="B2:E57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2" customWidth="1" style="77" min="1" max="1"/>
@@ -43696,6 +44622,126 @@
       <c r="E51" s="95" t="inlineStr">
         <is>
           <t>Expliquer ces chèques et leur traitement (item 91).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="72" customHeight="1" s="48">
+      <c r="B52" s="96" t="n">
+        <v>47</v>
+      </c>
+      <c r="C52" s="95" t="inlineStr">
+        <is>
+          <t>Comptes 2023 et 31/08/2026</t>
+        </is>
+      </c>
+      <c r="D52" s="95" t="inlineStr">
+        <is>
+          <t>Deux versions des comptes 2023 (écart de 10 000 000 FCFA sur l'actif brut et de 1 930 000 FCFA sur l'excédent) ; résultat au 31/08/2026 différent de 4 108 040 FCFA entre états financiers et balance.</t>
+        </is>
+      </c>
+      <c r="E52" s="95" t="inlineStr">
+        <is>
+          <t>Version approuvée et explication des écarts (item 110).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="72" customHeight="1" s="48">
+      <c r="B53" s="96" t="n">
+        <v>48</v>
+      </c>
+      <c r="C53" s="95" t="inlineStr">
+        <is>
+          <t>Clé maladie / décès avant mars 2024</t>
+        </is>
+      </c>
+      <c r="D53" s="95" t="inlineStr">
+        <is>
+          <t>En janvier et février 2024, le précompte décès ne vaut pas 1,23 / 3,77 du précompte maladie ; la clé 3,77 / 1,23 s'applique à plus de 99 % des lignes ensuite.</t>
+        </is>
+      </c>
+      <c r="E53" s="95" t="inlineStr">
+        <is>
+          <t>Clé appliquée et décision (item 111).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="72" customHeight="1" s="48">
+      <c r="B54" s="96" t="n">
+        <v>49</v>
+      </c>
+      <c r="C54" s="95" t="inlineStr">
+        <is>
+          <t>Épargne présentée en Assemblée générale</t>
+        </is>
+      </c>
+      <c r="D54" s="95" t="inlineStr">
+        <is>
+          <t>Le rapport de gestion 2025 présente la collecte de l'année (4 387 823 635 FCFA) comme l'épargne au 31/12/2025, alors que la dette d'épargne de la balance dépasse 13,8 milliards de FCFA.</t>
+        </is>
+      </c>
+      <c r="E54" s="95" t="inlineStr">
+        <is>
+          <t>Rapport rectifié (item 112).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="72" customHeight="1" s="48">
+      <c r="B55" s="96" t="n">
+        <v>50</v>
+      </c>
+      <c r="C55" s="95" t="inlineStr">
+        <is>
+          <t>Intérêts servis</t>
+        </is>
+      </c>
+      <c r="D55" s="95" t="inlineStr">
+        <is>
+          <t>Aucune écriture d'intérêts sur les comptes PEP et EFC dans le grand livre 2024 et aucun compte de charge d'intérêts servis dans les balances 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="E55" s="95" t="inlineStr">
+        <is>
+          <t>Indiquer comment les intérêts promis sont calculés et payés (items 18 et 99).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="60" customHeight="1" s="48">
+      <c r="B56" s="96" t="n">
+        <v>51</v>
+      </c>
+      <c r="C56" s="95" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="D56" s="95" t="inlineStr">
+        <is>
+          <t>Cinq salariés ont 55 ans ou plus en 2025 et restent en poste ; douze dates d'embauche changent dans la DISA 2025 ; dix-neuf recrues de 2025 sans entité.</t>
+        </is>
+      </c>
+      <c r="E56" s="95" t="inlineStr">
+        <is>
+          <t>Âge de départ, dates et entités (item 113).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1" s="48">
+      <c r="B57" s="96" t="n">
+        <v>52</v>
+      </c>
+      <c r="C57" s="95" t="inlineStr">
+        <is>
+          <t>Retraités</t>
+        </is>
+      </c>
+      <c r="D57" s="95" t="inlineStr">
+        <is>
+          <t>La convention IPS-CGRAE ne fixe pas la cotisation des retraités et interdit au FPPN de suspendre les soins en cas de retard de reversement.</t>
+        </is>
+      </c>
+      <c r="E57" s="95" t="inlineStr">
+        <is>
+          <t>Bulletin, barème et liste des non précomptés (item 114).</t>
         </is>
       </c>
     </row>

</xml_diff>